<commit_message>
Add Coteccons logo and real L&OD contact; host on GitHub Pages
- player/logo.png (white logo) is now the default header logo in every package
- brand/ keeps the original white and color logos
- Default out-of-attempts contact: Mr. Minh (minhvt02@coteccons.vn) or cta@coteccons.vn
- Regenerate Excel template; update HANDOFF, BUILDER_SPEC, CLAUDE.md
- Player tests: 26/26 pass

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DkjQ94JxW9pMDUqdRVGGx
</commit_message>
<xml_diff>
--- a/templates/Mau_nhap_lieu_khoa_hoc.xlsx
+++ b/templates/Mau_nhap_lieu_khoa_hoc.xlsx
@@ -956,7 +956,7 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Bạn đã dùng hết lượt làm bài. Vui lòng liên hệ L&amp;OD Team để được hỗ trợ đăng ký lại. (Thay bằng tên, email, số điện thoại đầu mối L&amp;OD)</t>
+          <t>Bạn đã dùng hết lượt làm bài. Vui lòng liên hệ L&amp;OD: Mr. Minh (minhvt02@coteccons.vn) hoặc cta@coteccons.vn để được hỗ trợ đăng ký lại.</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
@@ -974,7 +974,7 @@
       <c r="B11" s="8" t="inlineStr"/>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Tên file logo đặt trong thư mục khóa. Để trống = dùng chữ COTECCONS</t>
+          <t>Tên file logo đặt trong thư mục khóa. Để trống = dùng logo Coteccons trắng có sẵn</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Builder M1: pick files, read Excel + video folder, error check screen
- Split the Excel template: templates/Mau_nhap_lieu_khoa_hoc.xlsx is now a clean
  blank template for trainers (with exam-settings and pop-up writing tips);
  the demo course moves to demo-course/ATLD-DEMO.xlsx
- builder/: Vite + plain JS. xlsx.js reads .xlsx with fflate (no SheetJS);
  course.js mirrors build_scorm.py read_excel() and adds the checks from the
  spec (similar-name hints, pop-up past video end, course code, gaps, size)
- Unit tests compare course data with build_scorm.py and cover 5 error types;
  tests/test_builder.py drives the page in Chromium
- GitHub Actions: test + deploy Builder to GitHub Pages on main
- Docs updated (CLAUDE.md, README, HANDOFF, BUILDER_SPEC)

Tests: Player 26/26, Builder unit 6/6, Builder UI 17/17

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013DkjQ94JxW9pMDUqdRVGGx
</commit_message>
<xml_diff>
--- a/templates/Mau_nhap_lieu_khoa_hoc.xlsx
+++ b/templates/Mau_nhap_lieu_khoa_hoc.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,11 +140,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -526,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -776,13 +772,121 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Xáo phương án</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Thứ tự phương án được xáo mỗi lần thi. Dùng được 'Tất cả đều đúng', tránh viết 'Cả A và B đều đúng'</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Cài đặt bài kiểm tra (sheet 'Thông tin khóa')</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Gợi ý</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Điểm đạt 80% · 3 lượt · rút 15–20 câu từ ngân hàng 20–30 câu để mỗi lượt có đề khác nhau</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Gợi ý</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Thời gian làm bài: khoảng 1–1,5 phút cho mỗi câu. Hiện đáp án: nên chọn 'Không' để người rớt không học thuộc đáp án cho lượt sau</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Cách viết câu hỏi pop-up</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Mục đích là giữ học viên tập trung, không đánh đố. Hỏi đúng điều vừa nói trong 1–2 phút trước mốc</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Đặt mốc ngay sau khi ý chính kết thúc. Khoảng 1 câu cho mỗi 3–5 phút video, cách nhau ít nhất 1 phút</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Không đặt trong 30 giây đầu hoặc ở cuối video. 2–3 phương án ngắn là đủ. Nên có Giải thích</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Không dùng lại câu hỏi cuối khóa làm pop-up</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Ô cần điền</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n"/>
+      <c r="B37" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -826,11 +930,7 @@
           <t>Mã khóa</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
-        <is>
-          <t>ATLD-DEMO</t>
-        </is>
-      </c>
+      <c r="B2" s="8" t="inlineStr"/>
       <c r="C2" s="9" t="inlineStr">
         <is>
           <t>Không dấu, không khoảng trắng. Dùng làm tên file SCORM</t>
@@ -843,11 +943,7 @@
           <t>Tên khóa</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>An toàn lao động cơ bản (Demo)</t>
-        </is>
-      </c>
+      <c r="B3" s="8" t="inlineStr"/>
       <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Hiển thị trên đầu trang khóa học</t>
@@ -860,11 +956,7 @@
           <t>Mô tả ngắn</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Khóa demo minh họa các tính năng của Coteccons SCORM Player. Nội dung chỉ mang tính minh họa.</t>
-        </is>
-      </c>
+      <c r="B4" s="8" t="inlineStr"/>
       <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Dùng khi tạo khóa trên Workday</t>
@@ -908,7 +1000,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
@@ -923,7 +1015,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
@@ -939,7 +1031,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Có</t>
+          <t>Không</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1122,52 +1214,22 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Vì sao an toàn là trên hết</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>01_vi-sao-an-toan.mp4</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr"/>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Trang bị bảo hộ cá nhân (PPE)</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="inlineStr">
-        <is>
-          <t>02_bao-ho-ca-nhan.mp4</t>
-        </is>
-      </c>
-      <c r="D4" s="13" t="inlineStr"/>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Nhận diện mối nguy tại công trường</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="inlineStr">
-        <is>
-          <t>03_nhan-dien-moi-nguy.mp4</t>
-        </is>
-      </c>
-      <c r="D5" s="13" t="inlineStr"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -1580,7 +1642,7 @@
       <c r="B2" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="14" t="inlineStr">
+      <c r="C2" s="13" t="inlineStr">
         <is>
           <t>00:20</t>
         </is>
@@ -1614,409 +1676,129 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>POPUP</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
-        <is>
-          <t>00:15</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Theo video, điều gì được đặt lên hàng đầu tại công trường?</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Tiến độ</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>An toàn</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Chi phí</t>
-        </is>
-      </c>
-      <c r="H3" s="8" t="inlineStr"/>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>An toàn luôn được ưu tiên trước tiến độ và chi phí.</t>
-        </is>
-      </c>
+      <c r="A3" s="6" t="n"/>
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+      <c r="I3" s="6" t="n"/>
+      <c r="J3" s="6" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>POPUP</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>00:40</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Ai có trách nhiệm về an toàn tại công trường?</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ cán bộ an toàn</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ chỉ huy trưởng</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Tất cả mọi người</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr"/>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>An toàn là trách nhiệm của mỗi người.</t>
-        </is>
-      </c>
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+      <c r="J4" s="6" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>POPUP</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
-        <is>
-          <t>00:25</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>Mũ bảo hộ cần được đội như thế nào?</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Đội lỏng cho thoải mái</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Cài quai cằm chắc chắn</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Chỉ đội khi có người kiểm tra</t>
-        </is>
-      </c>
-      <c r="H5" s="8" t="inlineStr"/>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr"/>
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="14" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="6" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>POPUP</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>00:30</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Khi phát hiện mối nguy, việc đầu tiên nên làm là gì?</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Tiếp tục làm việc</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Báo ngay cho người phụ trách</t>
-        </is>
-      </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Tự xử lý một mình</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J6" s="8" t="inlineStr"/>
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
+      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr"/>
-      <c r="C7" s="15" t="inlineStr"/>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Mục đích chính của trang bị bảo hộ cá nhân là gì?</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Làm đẹp đồng phục</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Giảm nguy cơ chấn thương</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Thay thế biện pháp quản lý</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr"/>
-      <c r="I7" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>PPE là lớp bảo vệ cuối cùng, giúp giảm nguy cơ chấn thương.</t>
-        </is>
-      </c>
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
+      <c r="J7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr"/>
-      <c r="C8" s="15" t="inlineStr"/>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Khi thấy đồng nghiệp không đội mũ bảo hộ, bạn nên làm gì?</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Im lặng</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Nhắc nhở ngay</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Chụp ảnh đăng mạng xã hội</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>Báo cáo sau một tuần</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J8" s="8" t="inlineStr"/>
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr"/>
-      <c r="C9" s="15" t="inlineStr"/>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Phát hiện dây điện bị hở trên lối đi, bạn nên làm gì trước tiên?</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Bước qua và đi tiếp</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Rào chắn khu vực và báo người phụ trách</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>Tự nối lại dây điện</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr"/>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J9" s="8" t="inlineStr"/>
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr"/>
-      <c r="C10" s="15" t="inlineStr"/>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>An toàn lao động là trách nhiệm của ai?</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Riêng bộ phận an toàn</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Riêng ban chỉ huy</t>
-        </is>
-      </c>
-      <c r="G10" s="8" t="inlineStr">
-        <is>
-          <t>Mọi người trên công trường</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr"/>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="J10" s="8" t="inlineStr"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr"/>
-      <c r="C11" s="15" t="inlineStr"/>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Trước khi bắt đầu ca làm việc, bạn nên làm gì?</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Kiểm tra trang bị bảo hộ và khu vực làm việc</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Bắt đầu ngay để kịp tiến độ</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>Chờ có người nhắc</t>
-        </is>
-      </c>
-      <c r="H11" s="8" t="inlineStr"/>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="J11" s="8" t="inlineStr"/>
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>CUOI KHOA</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr"/>
-      <c r="C12" s="15" t="inlineStr"/>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Khi không chắc chắn về quy trình an toàn của một công việc, bạn nên?</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Làm theo cách mình nghĩ</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Hỏi người phụ trách trước khi làm</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
-        <is>
-          <t>Bỏ qua bước không rõ</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr"/>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr"/>
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="6" t="n"/>
-      <c r="C13" s="16" t="n"/>
+      <c r="C13" s="14" t="n"/>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
       <c r="F13" s="6" t="n"/>
@@ -2028,7 +1810,7 @@
     <row r="14">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="6" t="n"/>
-      <c r="C14" s="16" t="n"/>
+      <c r="C14" s="14" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
@@ -2040,7 +1822,7 @@
     <row r="15">
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="6" t="n"/>
-      <c r="C15" s="16" t="n"/>
+      <c r="C15" s="14" t="n"/>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
@@ -2052,7 +1834,7 @@
     <row r="16">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="6" t="n"/>
-      <c r="C16" s="16" t="n"/>
+      <c r="C16" s="14" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
@@ -2064,7 +1846,7 @@
     <row r="17">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="6" t="n"/>
-      <c r="C17" s="16" t="n"/>
+      <c r="C17" s="14" t="n"/>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
@@ -2076,7 +1858,7 @@
     <row r="18">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="6" t="n"/>
-      <c r="C18" s="16" t="n"/>
+      <c r="C18" s="14" t="n"/>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
@@ -2088,7 +1870,7 @@
     <row r="19">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="6" t="n"/>
-      <c r="C19" s="16" t="n"/>
+      <c r="C19" s="14" t="n"/>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
       <c r="F19" s="6" t="n"/>
@@ -2100,7 +1882,7 @@
     <row r="20">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="6" t="n"/>
-      <c r="C20" s="16" t="n"/>
+      <c r="C20" s="14" t="n"/>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
@@ -2112,7 +1894,7 @@
     <row r="21">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="6" t="n"/>
-      <c r="C21" s="16" t="n"/>
+      <c r="C21" s="14" t="n"/>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
@@ -2124,7 +1906,7 @@
     <row r="22">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="6" t="n"/>
-      <c r="C22" s="16" t="n"/>
+      <c r="C22" s="14" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
@@ -2136,7 +1918,7 @@
     <row r="23">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="6" t="n"/>
-      <c r="C23" s="16" t="n"/>
+      <c r="C23" s="14" t="n"/>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
@@ -2148,7 +1930,7 @@
     <row r="24">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="6" t="n"/>
-      <c r="C24" s="16" t="n"/>
+      <c r="C24" s="14" t="n"/>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
@@ -2160,7 +1942,7 @@
     <row r="25">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="6" t="n"/>
-      <c r="C25" s="16" t="n"/>
+      <c r="C25" s="14" t="n"/>
       <c r="D25" s="6" t="n"/>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
@@ -2172,7 +1954,7 @@
     <row r="26">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="6" t="n"/>
-      <c r="C26" s="16" t="n"/>
+      <c r="C26" s="14" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="n"/>
@@ -2184,7 +1966,7 @@
     <row r="27">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="6" t="n"/>
-      <c r="C27" s="16" t="n"/>
+      <c r="C27" s="14" t="n"/>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
@@ -2196,7 +1978,7 @@
     <row r="28">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="6" t="n"/>
-      <c r="C28" s="16" t="n"/>
+      <c r="C28" s="14" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="n"/>
       <c r="F28" s="6" t="n"/>
@@ -2208,7 +1990,7 @@
     <row r="29">
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="6" t="n"/>
-      <c r="C29" s="16" t="n"/>
+      <c r="C29" s="14" t="n"/>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
       <c r="F29" s="6" t="n"/>
@@ -2220,7 +2002,7 @@
     <row r="30">
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="6" t="n"/>
-      <c r="C30" s="16" t="n"/>
+      <c r="C30" s="14" t="n"/>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
       <c r="F30" s="6" t="n"/>
@@ -2232,7 +2014,7 @@
     <row r="31">
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="6" t="n"/>
-      <c r="C31" s="16" t="n"/>
+      <c r="C31" s="14" t="n"/>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
       <c r="F31" s="6" t="n"/>
@@ -2244,7 +2026,7 @@
     <row r="32">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="6" t="n"/>
-      <c r="C32" s="16" t="n"/>
+      <c r="C32" s="14" t="n"/>
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="6" t="n"/>
       <c r="F32" s="6" t="n"/>
@@ -2256,7 +2038,7 @@
     <row r="33">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="6" t="n"/>
-      <c r="C33" s="16" t="n"/>
+      <c r="C33" s="14" t="n"/>
       <c r="D33" s="6" t="n"/>
       <c r="E33" s="6" t="n"/>
       <c r="F33" s="6" t="n"/>
@@ -2268,7 +2050,7 @@
     <row r="34">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="6" t="n"/>
-      <c r="C34" s="16" t="n"/>
+      <c r="C34" s="14" t="n"/>
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="n"/>
       <c r="F34" s="6" t="n"/>
@@ -2280,7 +2062,7 @@
     <row r="35">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="6" t="n"/>
-      <c r="C35" s="16" t="n"/>
+      <c r="C35" s="14" t="n"/>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>
       <c r="F35" s="6" t="n"/>
@@ -2292,7 +2074,7 @@
     <row r="36">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="6" t="n"/>
-      <c r="C36" s="16" t="n"/>
+      <c r="C36" s="14" t="n"/>
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="n"/>
@@ -2304,7 +2086,7 @@
     <row r="37">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="n"/>
-      <c r="C37" s="16" t="n"/>
+      <c r="C37" s="14" t="n"/>
       <c r="D37" s="6" t="n"/>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="n"/>
@@ -2316,7 +2098,7 @@
     <row r="38">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6" t="n"/>
-      <c r="C38" s="16" t="n"/>
+      <c r="C38" s="14" t="n"/>
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="n"/>
       <c r="F38" s="6" t="n"/>
@@ -2328,7 +2110,7 @@
     <row r="39">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="n"/>
-      <c r="C39" s="16" t="n"/>
+      <c r="C39" s="14" t="n"/>
       <c r="D39" s="6" t="n"/>
       <c r="E39" s="6" t="n"/>
       <c r="F39" s="6" t="n"/>
@@ -2340,7 +2122,7 @@
     <row r="40">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="6" t="n"/>
-      <c r="C40" s="16" t="n"/>
+      <c r="C40" s="14" t="n"/>
       <c r="D40" s="6" t="n"/>
       <c r="E40" s="6" t="n"/>
       <c r="F40" s="6" t="n"/>
@@ -2352,7 +2134,7 @@
     <row r="41">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6" t="n"/>
-      <c r="C41" s="16" t="n"/>
+      <c r="C41" s="14" t="n"/>
       <c r="D41" s="6" t="n"/>
       <c r="E41" s="6" t="n"/>
       <c r="F41" s="6" t="n"/>
@@ -2364,7 +2146,7 @@
     <row r="42">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="6" t="n"/>
-      <c r="C42" s="16" t="n"/>
+      <c r="C42" s="14" t="n"/>
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="n"/>
       <c r="F42" s="6" t="n"/>
@@ -2376,7 +2158,7 @@
     <row r="43">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="6" t="n"/>
-      <c r="C43" s="16" t="n"/>
+      <c r="C43" s="14" t="n"/>
       <c r="D43" s="6" t="n"/>
       <c r="E43" s="6" t="n"/>
       <c r="F43" s="6" t="n"/>
@@ -2388,7 +2170,7 @@
     <row r="44">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="6" t="n"/>
-      <c r="C44" s="16" t="n"/>
+      <c r="C44" s="14" t="n"/>
       <c r="D44" s="6" t="n"/>
       <c r="E44" s="6" t="n"/>
       <c r="F44" s="6" t="n"/>
@@ -2400,7 +2182,7 @@
     <row r="45">
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="6" t="n"/>
-      <c r="C45" s="16" t="n"/>
+      <c r="C45" s="14" t="n"/>
       <c r="D45" s="6" t="n"/>
       <c r="E45" s="6" t="n"/>
       <c r="F45" s="6" t="n"/>
@@ -2412,7 +2194,7 @@
     <row r="46">
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="6" t="n"/>
-      <c r="C46" s="16" t="n"/>
+      <c r="C46" s="14" t="n"/>
       <c r="D46" s="6" t="n"/>
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="6" t="n"/>
@@ -2424,7 +2206,7 @@
     <row r="47">
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="6" t="n"/>
-      <c r="C47" s="16" t="n"/>
+      <c r="C47" s="14" t="n"/>
       <c r="D47" s="6" t="n"/>
       <c r="E47" s="6" t="n"/>
       <c r="F47" s="6" t="n"/>
@@ -2436,7 +2218,7 @@
     <row r="48">
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="6" t="n"/>
-      <c r="C48" s="16" t="n"/>
+      <c r="C48" s="14" t="n"/>
       <c r="D48" s="6" t="n"/>
       <c r="E48" s="6" t="n"/>
       <c r="F48" s="6" t="n"/>
@@ -2448,7 +2230,7 @@
     <row r="49">
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="6" t="n"/>
-      <c r="C49" s="16" t="n"/>
+      <c r="C49" s="14" t="n"/>
       <c r="D49" s="6" t="n"/>
       <c r="E49" s="6" t="n"/>
       <c r="F49" s="6" t="n"/>
@@ -2460,7 +2242,7 @@
     <row r="50">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="6" t="n"/>
-      <c r="C50" s="16" t="n"/>
+      <c r="C50" s="14" t="n"/>
       <c r="D50" s="6" t="n"/>
       <c r="E50" s="6" t="n"/>
       <c r="F50" s="6" t="n"/>
@@ -2472,7 +2254,7 @@
     <row r="51">
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="6" t="n"/>
-      <c r="C51" s="16" t="n"/>
+      <c r="C51" s="14" t="n"/>
       <c r="D51" s="6" t="n"/>
       <c r="E51" s="6" t="n"/>
       <c r="F51" s="6" t="n"/>
@@ -2484,7 +2266,7 @@
     <row r="52">
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="6" t="n"/>
-      <c r="C52" s="16" t="n"/>
+      <c r="C52" s="14" t="n"/>
       <c r="D52" s="6" t="n"/>
       <c r="E52" s="6" t="n"/>
       <c r="F52" s="6" t="n"/>
@@ -2496,7 +2278,7 @@
     <row r="53">
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="6" t="n"/>
-      <c r="C53" s="16" t="n"/>
+      <c r="C53" s="14" t="n"/>
       <c r="D53" s="6" t="n"/>
       <c r="E53" s="6" t="n"/>
       <c r="F53" s="6" t="n"/>
@@ -2508,7 +2290,7 @@
     <row r="54">
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="6" t="n"/>
-      <c r="C54" s="16" t="n"/>
+      <c r="C54" s="14" t="n"/>
       <c r="D54" s="6" t="n"/>
       <c r="E54" s="6" t="n"/>
       <c r="F54" s="6" t="n"/>
@@ -2520,7 +2302,7 @@
     <row r="55">
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="6" t="n"/>
-      <c r="C55" s="16" t="n"/>
+      <c r="C55" s="14" t="n"/>
       <c r="D55" s="6" t="n"/>
       <c r="E55" s="6" t="n"/>
       <c r="F55" s="6" t="n"/>
@@ -2532,7 +2314,7 @@
     <row r="56">
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="6" t="n"/>
-      <c r="C56" s="16" t="n"/>
+      <c r="C56" s="14" t="n"/>
       <c r="D56" s="6" t="n"/>
       <c r="E56" s="6" t="n"/>
       <c r="F56" s="6" t="n"/>
@@ -2544,7 +2326,7 @@
     <row r="57">
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="6" t="n"/>
-      <c r="C57" s="16" t="n"/>
+      <c r="C57" s="14" t="n"/>
       <c r="D57" s="6" t="n"/>
       <c r="E57" s="6" t="n"/>
       <c r="F57" s="6" t="n"/>
@@ -2556,7 +2338,7 @@
     <row r="58">
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="6" t="n"/>
-      <c r="C58" s="16" t="n"/>
+      <c r="C58" s="14" t="n"/>
       <c r="D58" s="6" t="n"/>
       <c r="E58" s="6" t="n"/>
       <c r="F58" s="6" t="n"/>
@@ -2568,7 +2350,7 @@
     <row r="59">
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="6" t="n"/>
-      <c r="C59" s="16" t="n"/>
+      <c r="C59" s="14" t="n"/>
       <c r="D59" s="6" t="n"/>
       <c r="E59" s="6" t="n"/>
       <c r="F59" s="6" t="n"/>
@@ -2580,7 +2362,7 @@
     <row r="60">
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="6" t="n"/>
-      <c r="C60" s="16" t="n"/>
+      <c r="C60" s="14" t="n"/>
       <c r="D60" s="6" t="n"/>
       <c r="E60" s="6" t="n"/>
       <c r="F60" s="6" t="n"/>
@@ -2592,7 +2374,7 @@
     <row r="61">
       <c r="A61" s="6" t="n"/>
       <c r="B61" s="6" t="n"/>
-      <c r="C61" s="16" t="n"/>
+      <c r="C61" s="14" t="n"/>
       <c r="D61" s="6" t="n"/>
       <c r="E61" s="6" t="n"/>
       <c r="F61" s="6" t="n"/>
@@ -2604,7 +2386,7 @@
     <row r="62">
       <c r="A62" s="6" t="n"/>
       <c r="B62" s="6" t="n"/>
-      <c r="C62" s="16" t="n"/>
+      <c r="C62" s="14" t="n"/>
       <c r="D62" s="6" t="n"/>
       <c r="E62" s="6" t="n"/>
       <c r="F62" s="6" t="n"/>
@@ -2616,7 +2398,7 @@
     <row r="63">
       <c r="A63" s="6" t="n"/>
       <c r="B63" s="6" t="n"/>
-      <c r="C63" s="16" t="n"/>
+      <c r="C63" s="14" t="n"/>
       <c r="D63" s="6" t="n"/>
       <c r="E63" s="6" t="n"/>
       <c r="F63" s="6" t="n"/>
@@ -2628,7 +2410,7 @@
     <row r="64">
       <c r="A64" s="6" t="n"/>
       <c r="B64" s="6" t="n"/>
-      <c r="C64" s="16" t="n"/>
+      <c r="C64" s="14" t="n"/>
       <c r="D64" s="6" t="n"/>
       <c r="E64" s="6" t="n"/>
       <c r="F64" s="6" t="n"/>
@@ -2640,7 +2422,7 @@
     <row r="65">
       <c r="A65" s="6" t="n"/>
       <c r="B65" s="6" t="n"/>
-      <c r="C65" s="16" t="n"/>
+      <c r="C65" s="14" t="n"/>
       <c r="D65" s="6" t="n"/>
       <c r="E65" s="6" t="n"/>
       <c r="F65" s="6" t="n"/>
@@ -2652,7 +2434,7 @@
     <row r="66">
       <c r="A66" s="6" t="n"/>
       <c r="B66" s="6" t="n"/>
-      <c r="C66" s="16" t="n"/>
+      <c r="C66" s="14" t="n"/>
       <c r="D66" s="6" t="n"/>
       <c r="E66" s="6" t="n"/>
       <c r="F66" s="6" t="n"/>
@@ -2664,7 +2446,7 @@
     <row r="67">
       <c r="A67" s="6" t="n"/>
       <c r="B67" s="6" t="n"/>
-      <c r="C67" s="16" t="n"/>
+      <c r="C67" s="14" t="n"/>
       <c r="D67" s="6" t="n"/>
       <c r="E67" s="6" t="n"/>
       <c r="F67" s="6" t="n"/>
@@ -2676,7 +2458,7 @@
     <row r="68">
       <c r="A68" s="6" t="n"/>
       <c r="B68" s="6" t="n"/>
-      <c r="C68" s="16" t="n"/>
+      <c r="C68" s="14" t="n"/>
       <c r="D68" s="6" t="n"/>
       <c r="E68" s="6" t="n"/>
       <c r="F68" s="6" t="n"/>
@@ -2688,7 +2470,7 @@
     <row r="69">
       <c r="A69" s="6" t="n"/>
       <c r="B69" s="6" t="n"/>
-      <c r="C69" s="16" t="n"/>
+      <c r="C69" s="14" t="n"/>
       <c r="D69" s="6" t="n"/>
       <c r="E69" s="6" t="n"/>
       <c r="F69" s="6" t="n"/>
@@ -2700,7 +2482,7 @@
     <row r="70">
       <c r="A70" s="6" t="n"/>
       <c r="B70" s="6" t="n"/>
-      <c r="C70" s="16" t="n"/>
+      <c r="C70" s="14" t="n"/>
       <c r="D70" s="6" t="n"/>
       <c r="E70" s="6" t="n"/>
       <c r="F70" s="6" t="n"/>
@@ -2712,7 +2494,7 @@
     <row r="71">
       <c r="A71" s="6" t="n"/>
       <c r="B71" s="6" t="n"/>
-      <c r="C71" s="16" t="n"/>
+      <c r="C71" s="14" t="n"/>
       <c r="D71" s="6" t="n"/>
       <c r="E71" s="6" t="n"/>
       <c r="F71" s="6" t="n"/>
@@ -2724,7 +2506,7 @@
     <row r="72">
       <c r="A72" s="6" t="n"/>
       <c r="B72" s="6" t="n"/>
-      <c r="C72" s="16" t="n"/>
+      <c r="C72" s="14" t="n"/>
       <c r="D72" s="6" t="n"/>
       <c r="E72" s="6" t="n"/>
       <c r="F72" s="6" t="n"/>
@@ -2736,7 +2518,7 @@
     <row r="73">
       <c r="A73" s="6" t="n"/>
       <c r="B73" s="6" t="n"/>
-      <c r="C73" s="16" t="n"/>
+      <c r="C73" s="14" t="n"/>
       <c r="D73" s="6" t="n"/>
       <c r="E73" s="6" t="n"/>
       <c r="F73" s="6" t="n"/>
@@ -2748,7 +2530,7 @@
     <row r="74">
       <c r="A74" s="6" t="n"/>
       <c r="B74" s="6" t="n"/>
-      <c r="C74" s="16" t="n"/>
+      <c r="C74" s="14" t="n"/>
       <c r="D74" s="6" t="n"/>
       <c r="E74" s="6" t="n"/>
       <c r="F74" s="6" t="n"/>
@@ -2760,7 +2542,7 @@
     <row r="75">
       <c r="A75" s="6" t="n"/>
       <c r="B75" s="6" t="n"/>
-      <c r="C75" s="16" t="n"/>
+      <c r="C75" s="14" t="n"/>
       <c r="D75" s="6" t="n"/>
       <c r="E75" s="6" t="n"/>
       <c r="F75" s="6" t="n"/>
@@ -2772,7 +2554,7 @@
     <row r="76">
       <c r="A76" s="6" t="n"/>
       <c r="B76" s="6" t="n"/>
-      <c r="C76" s="16" t="n"/>
+      <c r="C76" s="14" t="n"/>
       <c r="D76" s="6" t="n"/>
       <c r="E76" s="6" t="n"/>
       <c r="F76" s="6" t="n"/>
@@ -2784,7 +2566,7 @@
     <row r="77">
       <c r="A77" s="6" t="n"/>
       <c r="B77" s="6" t="n"/>
-      <c r="C77" s="16" t="n"/>
+      <c r="C77" s="14" t="n"/>
       <c r="D77" s="6" t="n"/>
       <c r="E77" s="6" t="n"/>
       <c r="F77" s="6" t="n"/>
@@ -2796,7 +2578,7 @@
     <row r="78">
       <c r="A78" s="6" t="n"/>
       <c r="B78" s="6" t="n"/>
-      <c r="C78" s="16" t="n"/>
+      <c r="C78" s="14" t="n"/>
       <c r="D78" s="6" t="n"/>
       <c r="E78" s="6" t="n"/>
       <c r="F78" s="6" t="n"/>
@@ -2808,7 +2590,7 @@
     <row r="79">
       <c r="A79" s="6" t="n"/>
       <c r="B79" s="6" t="n"/>
-      <c r="C79" s="16" t="n"/>
+      <c r="C79" s="14" t="n"/>
       <c r="D79" s="6" t="n"/>
       <c r="E79" s="6" t="n"/>
       <c r="F79" s="6" t="n"/>
@@ -2820,7 +2602,7 @@
     <row r="80">
       <c r="A80" s="6" t="n"/>
       <c r="B80" s="6" t="n"/>
-      <c r="C80" s="16" t="n"/>
+      <c r="C80" s="14" t="n"/>
       <c r="D80" s="6" t="n"/>
       <c r="E80" s="6" t="n"/>
       <c r="F80" s="6" t="n"/>
@@ -2832,7 +2614,7 @@
     <row r="81">
       <c r="A81" s="6" t="n"/>
       <c r="B81" s="6" t="n"/>
-      <c r="C81" s="16" t="n"/>
+      <c r="C81" s="14" t="n"/>
       <c r="D81" s="6" t="n"/>
       <c r="E81" s="6" t="n"/>
       <c r="F81" s="6" t="n"/>
@@ -2844,7 +2626,7 @@
     <row r="82">
       <c r="A82" s="6" t="n"/>
       <c r="B82" s="6" t="n"/>
-      <c r="C82" s="16" t="n"/>
+      <c r="C82" s="14" t="n"/>
       <c r="D82" s="6" t="n"/>
       <c r="E82" s="6" t="n"/>
       <c r="F82" s="6" t="n"/>
@@ -2856,7 +2638,7 @@
     <row r="83">
       <c r="A83" s="6" t="n"/>
       <c r="B83" s="6" t="n"/>
-      <c r="C83" s="16" t="n"/>
+      <c r="C83" s="14" t="n"/>
       <c r="D83" s="6" t="n"/>
       <c r="E83" s="6" t="n"/>
       <c r="F83" s="6" t="n"/>
@@ -2868,7 +2650,7 @@
     <row r="84">
       <c r="A84" s="6" t="n"/>
       <c r="B84" s="6" t="n"/>
-      <c r="C84" s="16" t="n"/>
+      <c r="C84" s="14" t="n"/>
       <c r="D84" s="6" t="n"/>
       <c r="E84" s="6" t="n"/>
       <c r="F84" s="6" t="n"/>
@@ -2880,7 +2662,7 @@
     <row r="85">
       <c r="A85" s="6" t="n"/>
       <c r="B85" s="6" t="n"/>
-      <c r="C85" s="16" t="n"/>
+      <c r="C85" s="14" t="n"/>
       <c r="D85" s="6" t="n"/>
       <c r="E85" s="6" t="n"/>
       <c r="F85" s="6" t="n"/>
@@ -2892,7 +2674,7 @@
     <row r="86">
       <c r="A86" s="6" t="n"/>
       <c r="B86" s="6" t="n"/>
-      <c r="C86" s="16" t="n"/>
+      <c r="C86" s="14" t="n"/>
       <c r="D86" s="6" t="n"/>
       <c r="E86" s="6" t="n"/>
       <c r="F86" s="6" t="n"/>
@@ -2904,7 +2686,7 @@
     <row r="87">
       <c r="A87" s="6" t="n"/>
       <c r="B87" s="6" t="n"/>
-      <c r="C87" s="16" t="n"/>
+      <c r="C87" s="14" t="n"/>
       <c r="D87" s="6" t="n"/>
       <c r="E87" s="6" t="n"/>
       <c r="F87" s="6" t="n"/>
@@ -2916,7 +2698,7 @@
     <row r="88">
       <c r="A88" s="6" t="n"/>
       <c r="B88" s="6" t="n"/>
-      <c r="C88" s="16" t="n"/>
+      <c r="C88" s="14" t="n"/>
       <c r="D88" s="6" t="n"/>
       <c r="E88" s="6" t="n"/>
       <c r="F88" s="6" t="n"/>
@@ -2928,7 +2710,7 @@
     <row r="89">
       <c r="A89" s="6" t="n"/>
       <c r="B89" s="6" t="n"/>
-      <c r="C89" s="16" t="n"/>
+      <c r="C89" s="14" t="n"/>
       <c r="D89" s="6" t="n"/>
       <c r="E89" s="6" t="n"/>
       <c r="F89" s="6" t="n"/>
@@ -2940,7 +2722,7 @@
     <row r="90">
       <c r="A90" s="6" t="n"/>
       <c r="B90" s="6" t="n"/>
-      <c r="C90" s="16" t="n"/>
+      <c r="C90" s="14" t="n"/>
       <c r="D90" s="6" t="n"/>
       <c r="E90" s="6" t="n"/>
       <c r="F90" s="6" t="n"/>
@@ -2952,7 +2734,7 @@
     <row r="91">
       <c r="A91" s="6" t="n"/>
       <c r="B91" s="6" t="n"/>
-      <c r="C91" s="16" t="n"/>
+      <c r="C91" s="14" t="n"/>
       <c r="D91" s="6" t="n"/>
       <c r="E91" s="6" t="n"/>
       <c r="F91" s="6" t="n"/>
@@ -2964,7 +2746,7 @@
     <row r="92">
       <c r="A92" s="6" t="n"/>
       <c r="B92" s="6" t="n"/>
-      <c r="C92" s="16" t="n"/>
+      <c r="C92" s="14" t="n"/>
       <c r="D92" s="6" t="n"/>
       <c r="E92" s="6" t="n"/>
       <c r="F92" s="6" t="n"/>
@@ -2976,7 +2758,7 @@
     <row r="93">
       <c r="A93" s="6" t="n"/>
       <c r="B93" s="6" t="n"/>
-      <c r="C93" s="16" t="n"/>
+      <c r="C93" s="14" t="n"/>
       <c r="D93" s="6" t="n"/>
       <c r="E93" s="6" t="n"/>
       <c r="F93" s="6" t="n"/>
@@ -2988,7 +2770,7 @@
     <row r="94">
       <c r="A94" s="6" t="n"/>
       <c r="B94" s="6" t="n"/>
-      <c r="C94" s="16" t="n"/>
+      <c r="C94" s="14" t="n"/>
       <c r="D94" s="6" t="n"/>
       <c r="E94" s="6" t="n"/>
       <c r="F94" s="6" t="n"/>
@@ -3000,7 +2782,7 @@
     <row r="95">
       <c r="A95" s="6" t="n"/>
       <c r="B95" s="6" t="n"/>
-      <c r="C95" s="16" t="n"/>
+      <c r="C95" s="14" t="n"/>
       <c r="D95" s="6" t="n"/>
       <c r="E95" s="6" t="n"/>
       <c r="F95" s="6" t="n"/>
@@ -3012,7 +2794,7 @@
     <row r="96">
       <c r="A96" s="6" t="n"/>
       <c r="B96" s="6" t="n"/>
-      <c r="C96" s="16" t="n"/>
+      <c r="C96" s="14" t="n"/>
       <c r="D96" s="6" t="n"/>
       <c r="E96" s="6" t="n"/>
       <c r="F96" s="6" t="n"/>
@@ -3024,7 +2806,7 @@
     <row r="97">
       <c r="A97" s="6" t="n"/>
       <c r="B97" s="6" t="n"/>
-      <c r="C97" s="16" t="n"/>
+      <c r="C97" s="14" t="n"/>
       <c r="D97" s="6" t="n"/>
       <c r="E97" s="6" t="n"/>
       <c r="F97" s="6" t="n"/>
@@ -3036,7 +2818,7 @@
     <row r="98">
       <c r="A98" s="6" t="n"/>
       <c r="B98" s="6" t="n"/>
-      <c r="C98" s="16" t="n"/>
+      <c r="C98" s="14" t="n"/>
       <c r="D98" s="6" t="n"/>
       <c r="E98" s="6" t="n"/>
       <c r="F98" s="6" t="n"/>
@@ -3048,7 +2830,7 @@
     <row r="99">
       <c r="A99" s="6" t="n"/>
       <c r="B99" s="6" t="n"/>
-      <c r="C99" s="16" t="n"/>
+      <c r="C99" s="14" t="n"/>
       <c r="D99" s="6" t="n"/>
       <c r="E99" s="6" t="n"/>
       <c r="F99" s="6" t="n"/>
@@ -3060,7 +2842,7 @@
     <row r="100">
       <c r="A100" s="6" t="n"/>
       <c r="B100" s="6" t="n"/>
-      <c r="C100" s="16" t="n"/>
+      <c r="C100" s="14" t="n"/>
       <c r="D100" s="6" t="n"/>
       <c r="E100" s="6" t="n"/>
       <c r="F100" s="6" t="n"/>
@@ -3072,7 +2854,7 @@
     <row r="101">
       <c r="A101" s="6" t="n"/>
       <c r="B101" s="6" t="n"/>
-      <c r="C101" s="16" t="n"/>
+      <c r="C101" s="14" t="n"/>
       <c r="D101" s="6" t="n"/>
       <c r="E101" s="6" t="n"/>
       <c r="F101" s="6" t="n"/>
@@ -3084,7 +2866,7 @@
     <row r="102">
       <c r="A102" s="6" t="n"/>
       <c r="B102" s="6" t="n"/>
-      <c r="C102" s="16" t="n"/>
+      <c r="C102" s="14" t="n"/>
       <c r="D102" s="6" t="n"/>
       <c r="E102" s="6" t="n"/>
       <c r="F102" s="6" t="n"/>
@@ -3096,7 +2878,7 @@
     <row r="103">
       <c r="A103" s="6" t="n"/>
       <c r="B103" s="6" t="n"/>
-      <c r="C103" s="16" t="n"/>
+      <c r="C103" s="14" t="n"/>
       <c r="D103" s="6" t="n"/>
       <c r="E103" s="6" t="n"/>
       <c r="F103" s="6" t="n"/>
@@ -3108,7 +2890,7 @@
     <row r="104">
       <c r="A104" s="6" t="n"/>
       <c r="B104" s="6" t="n"/>
-      <c r="C104" s="16" t="n"/>
+      <c r="C104" s="14" t="n"/>
       <c r="D104" s="6" t="n"/>
       <c r="E104" s="6" t="n"/>
       <c r="F104" s="6" t="n"/>
@@ -3120,7 +2902,7 @@
     <row r="105">
       <c r="A105" s="6" t="n"/>
       <c r="B105" s="6" t="n"/>
-      <c r="C105" s="16" t="n"/>
+      <c r="C105" s="14" t="n"/>
       <c r="D105" s="6" t="n"/>
       <c r="E105" s="6" t="n"/>
       <c r="F105" s="6" t="n"/>
@@ -3132,7 +2914,7 @@
     <row r="106">
       <c r="A106" s="6" t="n"/>
       <c r="B106" s="6" t="n"/>
-      <c r="C106" s="16" t="n"/>
+      <c r="C106" s="14" t="n"/>
       <c r="D106" s="6" t="n"/>
       <c r="E106" s="6" t="n"/>
       <c r="F106" s="6" t="n"/>
@@ -3144,7 +2926,7 @@
     <row r="107">
       <c r="A107" s="6" t="n"/>
       <c r="B107" s="6" t="n"/>
-      <c r="C107" s="16" t="n"/>
+      <c r="C107" s="14" t="n"/>
       <c r="D107" s="6" t="n"/>
       <c r="E107" s="6" t="n"/>
       <c r="F107" s="6" t="n"/>
@@ -3156,7 +2938,7 @@
     <row r="108">
       <c r="A108" s="6" t="n"/>
       <c r="B108" s="6" t="n"/>
-      <c r="C108" s="16" t="n"/>
+      <c r="C108" s="14" t="n"/>
       <c r="D108" s="6" t="n"/>
       <c r="E108" s="6" t="n"/>
       <c r="F108" s="6" t="n"/>
@@ -3168,7 +2950,7 @@
     <row r="109">
       <c r="A109" s="6" t="n"/>
       <c r="B109" s="6" t="n"/>
-      <c r="C109" s="16" t="n"/>
+      <c r="C109" s="14" t="n"/>
       <c r="D109" s="6" t="n"/>
       <c r="E109" s="6" t="n"/>
       <c r="F109" s="6" t="n"/>
@@ -3180,7 +2962,7 @@
     <row r="110">
       <c r="A110" s="6" t="n"/>
       <c r="B110" s="6" t="n"/>
-      <c r="C110" s="16" t="n"/>
+      <c r="C110" s="14" t="n"/>
       <c r="D110" s="6" t="n"/>
       <c r="E110" s="6" t="n"/>
       <c r="F110" s="6" t="n"/>
@@ -3192,7 +2974,7 @@
     <row r="111">
       <c r="A111" s="6" t="n"/>
       <c r="B111" s="6" t="n"/>
-      <c r="C111" s="16" t="n"/>
+      <c r="C111" s="14" t="n"/>
       <c r="D111" s="6" t="n"/>
       <c r="E111" s="6" t="n"/>
       <c r="F111" s="6" t="n"/>
@@ -3204,7 +2986,7 @@
     <row r="112">
       <c r="A112" s="6" t="n"/>
       <c r="B112" s="6" t="n"/>
-      <c r="C112" s="16" t="n"/>
+      <c r="C112" s="14" t="n"/>
       <c r="D112" s="6" t="n"/>
       <c r="E112" s="6" t="n"/>
       <c r="F112" s="6" t="n"/>
@@ -3216,7 +2998,7 @@
     <row r="113">
       <c r="A113" s="6" t="n"/>
       <c r="B113" s="6" t="n"/>
-      <c r="C113" s="16" t="n"/>
+      <c r="C113" s="14" t="n"/>
       <c r="D113" s="6" t="n"/>
       <c r="E113" s="6" t="n"/>
       <c r="F113" s="6" t="n"/>
@@ -3228,7 +3010,7 @@
     <row r="114">
       <c r="A114" s="6" t="n"/>
       <c r="B114" s="6" t="n"/>
-      <c r="C114" s="16" t="n"/>
+      <c r="C114" s="14" t="n"/>
       <c r="D114" s="6" t="n"/>
       <c r="E114" s="6" t="n"/>
       <c r="F114" s="6" t="n"/>
@@ -3240,7 +3022,7 @@
     <row r="115">
       <c r="A115" s="6" t="n"/>
       <c r="B115" s="6" t="n"/>
-      <c r="C115" s="16" t="n"/>
+      <c r="C115" s="14" t="n"/>
       <c r="D115" s="6" t="n"/>
       <c r="E115" s="6" t="n"/>
       <c r="F115" s="6" t="n"/>
@@ -3252,7 +3034,7 @@
     <row r="116">
       <c r="A116" s="6" t="n"/>
       <c r="B116" s="6" t="n"/>
-      <c r="C116" s="16" t="n"/>
+      <c r="C116" s="14" t="n"/>
       <c r="D116" s="6" t="n"/>
       <c r="E116" s="6" t="n"/>
       <c r="F116" s="6" t="n"/>
@@ -3264,7 +3046,7 @@
     <row r="117">
       <c r="A117" s="6" t="n"/>
       <c r="B117" s="6" t="n"/>
-      <c r="C117" s="16" t="n"/>
+      <c r="C117" s="14" t="n"/>
       <c r="D117" s="6" t="n"/>
       <c r="E117" s="6" t="n"/>
       <c r="F117" s="6" t="n"/>
@@ -3276,7 +3058,7 @@
     <row r="118">
       <c r="A118" s="6" t="n"/>
       <c r="B118" s="6" t="n"/>
-      <c r="C118" s="16" t="n"/>
+      <c r="C118" s="14" t="n"/>
       <c r="D118" s="6" t="n"/>
       <c r="E118" s="6" t="n"/>
       <c r="F118" s="6" t="n"/>
@@ -3288,7 +3070,7 @@
     <row r="119">
       <c r="A119" s="6" t="n"/>
       <c r="B119" s="6" t="n"/>
-      <c r="C119" s="16" t="n"/>
+      <c r="C119" s="14" t="n"/>
       <c r="D119" s="6" t="n"/>
       <c r="E119" s="6" t="n"/>
       <c r="F119" s="6" t="n"/>
@@ -3300,7 +3082,7 @@
     <row r="120">
       <c r="A120" s="6" t="n"/>
       <c r="B120" s="6" t="n"/>
-      <c r="C120" s="16" t="n"/>
+      <c r="C120" s="14" t="n"/>
       <c r="D120" s="6" t="n"/>
       <c r="E120" s="6" t="n"/>
       <c r="F120" s="6" t="n"/>
@@ -3312,7 +3094,7 @@
     <row r="121">
       <c r="A121" s="6" t="n"/>
       <c r="B121" s="6" t="n"/>
-      <c r="C121" s="16" t="n"/>
+      <c r="C121" s="14" t="n"/>
       <c r="D121" s="6" t="n"/>
       <c r="E121" s="6" t="n"/>
       <c r="F121" s="6" t="n"/>
@@ -3324,7 +3106,7 @@
     <row r="122">
       <c r="A122" s="6" t="n"/>
       <c r="B122" s="6" t="n"/>
-      <c r="C122" s="16" t="n"/>
+      <c r="C122" s="14" t="n"/>
       <c r="D122" s="6" t="n"/>
       <c r="E122" s="6" t="n"/>
       <c r="F122" s="6" t="n"/>
@@ -3336,7 +3118,7 @@
     <row r="123">
       <c r="A123" s="6" t="n"/>
       <c r="B123" s="6" t="n"/>
-      <c r="C123" s="16" t="n"/>
+      <c r="C123" s="14" t="n"/>
       <c r="D123" s="6" t="n"/>
       <c r="E123" s="6" t="n"/>
       <c r="F123" s="6" t="n"/>
@@ -3348,7 +3130,7 @@
     <row r="124">
       <c r="A124" s="6" t="n"/>
       <c r="B124" s="6" t="n"/>
-      <c r="C124" s="16" t="n"/>
+      <c r="C124" s="14" t="n"/>
       <c r="D124" s="6" t="n"/>
       <c r="E124" s="6" t="n"/>
       <c r="F124" s="6" t="n"/>
@@ -3360,7 +3142,7 @@
     <row r="125">
       <c r="A125" s="6" t="n"/>
       <c r="B125" s="6" t="n"/>
-      <c r="C125" s="16" t="n"/>
+      <c r="C125" s="14" t="n"/>
       <c r="D125" s="6" t="n"/>
       <c r="E125" s="6" t="n"/>
       <c r="F125" s="6" t="n"/>
@@ -3372,7 +3154,7 @@
     <row r="126">
       <c r="A126" s="6" t="n"/>
       <c r="B126" s="6" t="n"/>
-      <c r="C126" s="16" t="n"/>
+      <c r="C126" s="14" t="n"/>
       <c r="D126" s="6" t="n"/>
       <c r="E126" s="6" t="n"/>
       <c r="F126" s="6" t="n"/>
@@ -3384,7 +3166,7 @@
     <row r="127">
       <c r="A127" s="6" t="n"/>
       <c r="B127" s="6" t="n"/>
-      <c r="C127" s="16" t="n"/>
+      <c r="C127" s="14" t="n"/>
       <c r="D127" s="6" t="n"/>
       <c r="E127" s="6" t="n"/>
       <c r="F127" s="6" t="n"/>
@@ -3396,7 +3178,7 @@
     <row r="128">
       <c r="A128" s="6" t="n"/>
       <c r="B128" s="6" t="n"/>
-      <c r="C128" s="16" t="n"/>
+      <c r="C128" s="14" t="n"/>
       <c r="D128" s="6" t="n"/>
       <c r="E128" s="6" t="n"/>
       <c r="F128" s="6" t="n"/>
@@ -3408,7 +3190,7 @@
     <row r="129">
       <c r="A129" s="6" t="n"/>
       <c r="B129" s="6" t="n"/>
-      <c r="C129" s="16" t="n"/>
+      <c r="C129" s="14" t="n"/>
       <c r="D129" s="6" t="n"/>
       <c r="E129" s="6" t="n"/>
       <c r="F129" s="6" t="n"/>
@@ -3420,7 +3202,7 @@
     <row r="130">
       <c r="A130" s="6" t="n"/>
       <c r="B130" s="6" t="n"/>
-      <c r="C130" s="16" t="n"/>
+      <c r="C130" s="14" t="n"/>
       <c r="D130" s="6" t="n"/>
       <c r="E130" s="6" t="n"/>
       <c r="F130" s="6" t="n"/>
@@ -3432,7 +3214,7 @@
     <row r="131">
       <c r="A131" s="6" t="n"/>
       <c r="B131" s="6" t="n"/>
-      <c r="C131" s="16" t="n"/>
+      <c r="C131" s="14" t="n"/>
       <c r="D131" s="6" t="n"/>
       <c r="E131" s="6" t="n"/>
       <c r="F131" s="6" t="n"/>
@@ -3444,7 +3226,7 @@
     <row r="132">
       <c r="A132" s="6" t="n"/>
       <c r="B132" s="6" t="n"/>
-      <c r="C132" s="16" t="n"/>
+      <c r="C132" s="14" t="n"/>
       <c r="D132" s="6" t="n"/>
       <c r="E132" s="6" t="n"/>
       <c r="F132" s="6" t="n"/>
@@ -3456,7 +3238,7 @@
     <row r="133">
       <c r="A133" s="6" t="n"/>
       <c r="B133" s="6" t="n"/>
-      <c r="C133" s="16" t="n"/>
+      <c r="C133" s="14" t="n"/>
       <c r="D133" s="6" t="n"/>
       <c r="E133" s="6" t="n"/>
       <c r="F133" s="6" t="n"/>
@@ -3468,7 +3250,7 @@
     <row r="134">
       <c r="A134" s="6" t="n"/>
       <c r="B134" s="6" t="n"/>
-      <c r="C134" s="16" t="n"/>
+      <c r="C134" s="14" t="n"/>
       <c r="D134" s="6" t="n"/>
       <c r="E134" s="6" t="n"/>
       <c r="F134" s="6" t="n"/>
@@ -3480,7 +3262,7 @@
     <row r="135">
       <c r="A135" s="6" t="n"/>
       <c r="B135" s="6" t="n"/>
-      <c r="C135" s="16" t="n"/>
+      <c r="C135" s="14" t="n"/>
       <c r="D135" s="6" t="n"/>
       <c r="E135" s="6" t="n"/>
       <c r="F135" s="6" t="n"/>
@@ -3492,7 +3274,7 @@
     <row r="136">
       <c r="A136" s="6" t="n"/>
       <c r="B136" s="6" t="n"/>
-      <c r="C136" s="16" t="n"/>
+      <c r="C136" s="14" t="n"/>
       <c r="D136" s="6" t="n"/>
       <c r="E136" s="6" t="n"/>
       <c r="F136" s="6" t="n"/>
@@ -3504,7 +3286,7 @@
     <row r="137">
       <c r="A137" s="6" t="n"/>
       <c r="B137" s="6" t="n"/>
-      <c r="C137" s="16" t="n"/>
+      <c r="C137" s="14" t="n"/>
       <c r="D137" s="6" t="n"/>
       <c r="E137" s="6" t="n"/>
       <c r="F137" s="6" t="n"/>
@@ -3516,7 +3298,7 @@
     <row r="138">
       <c r="A138" s="6" t="n"/>
       <c r="B138" s="6" t="n"/>
-      <c r="C138" s="16" t="n"/>
+      <c r="C138" s="14" t="n"/>
       <c r="D138" s="6" t="n"/>
       <c r="E138" s="6" t="n"/>
       <c r="F138" s="6" t="n"/>
@@ -3528,7 +3310,7 @@
     <row r="139">
       <c r="A139" s="6" t="n"/>
       <c r="B139" s="6" t="n"/>
-      <c r="C139" s="16" t="n"/>
+      <c r="C139" s="14" t="n"/>
       <c r="D139" s="6" t="n"/>
       <c r="E139" s="6" t="n"/>
       <c r="F139" s="6" t="n"/>
@@ -3540,7 +3322,7 @@
     <row r="140">
       <c r="A140" s="6" t="n"/>
       <c r="B140" s="6" t="n"/>
-      <c r="C140" s="16" t="n"/>
+      <c r="C140" s="14" t="n"/>
       <c r="D140" s="6" t="n"/>
       <c r="E140" s="6" t="n"/>
       <c r="F140" s="6" t="n"/>
@@ -3552,7 +3334,7 @@
     <row r="141">
       <c r="A141" s="6" t="n"/>
       <c r="B141" s="6" t="n"/>
-      <c r="C141" s="16" t="n"/>
+      <c r="C141" s="14" t="n"/>
       <c r="D141" s="6" t="n"/>
       <c r="E141" s="6" t="n"/>
       <c r="F141" s="6" t="n"/>
@@ -3564,7 +3346,7 @@
     <row r="142">
       <c r="A142" s="6" t="n"/>
       <c r="B142" s="6" t="n"/>
-      <c r="C142" s="16" t="n"/>
+      <c r="C142" s="14" t="n"/>
       <c r="D142" s="6" t="n"/>
       <c r="E142" s="6" t="n"/>
       <c r="F142" s="6" t="n"/>
@@ -3576,7 +3358,7 @@
     <row r="143">
       <c r="A143" s="6" t="n"/>
       <c r="B143" s="6" t="n"/>
-      <c r="C143" s="16" t="n"/>
+      <c r="C143" s="14" t="n"/>
       <c r="D143" s="6" t="n"/>
       <c r="E143" s="6" t="n"/>
       <c r="F143" s="6" t="n"/>
@@ -3588,7 +3370,7 @@
     <row r="144">
       <c r="A144" s="6" t="n"/>
       <c r="B144" s="6" t="n"/>
-      <c r="C144" s="16" t="n"/>
+      <c r="C144" s="14" t="n"/>
       <c r="D144" s="6" t="n"/>
       <c r="E144" s="6" t="n"/>
       <c r="F144" s="6" t="n"/>
@@ -3600,7 +3382,7 @@
     <row r="145">
       <c r="A145" s="6" t="n"/>
       <c r="B145" s="6" t="n"/>
-      <c r="C145" s="16" t="n"/>
+      <c r="C145" s="14" t="n"/>
       <c r="D145" s="6" t="n"/>
       <c r="E145" s="6" t="n"/>
       <c r="F145" s="6" t="n"/>
@@ -3612,7 +3394,7 @@
     <row r="146">
       <c r="A146" s="6" t="n"/>
       <c r="B146" s="6" t="n"/>
-      <c r="C146" s="16" t="n"/>
+      <c r="C146" s="14" t="n"/>
       <c r="D146" s="6" t="n"/>
       <c r="E146" s="6" t="n"/>
       <c r="F146" s="6" t="n"/>
@@ -3624,7 +3406,7 @@
     <row r="147">
       <c r="A147" s="6" t="n"/>
       <c r="B147" s="6" t="n"/>
-      <c r="C147" s="16" t="n"/>
+      <c r="C147" s="14" t="n"/>
       <c r="D147" s="6" t="n"/>
       <c r="E147" s="6" t="n"/>
       <c r="F147" s="6" t="n"/>
@@ -3636,7 +3418,7 @@
     <row r="148">
       <c r="A148" s="6" t="n"/>
       <c r="B148" s="6" t="n"/>
-      <c r="C148" s="16" t="n"/>
+      <c r="C148" s="14" t="n"/>
       <c r="D148" s="6" t="n"/>
       <c r="E148" s="6" t="n"/>
       <c r="F148" s="6" t="n"/>
@@ -3648,7 +3430,7 @@
     <row r="149">
       <c r="A149" s="6" t="n"/>
       <c r="B149" s="6" t="n"/>
-      <c r="C149" s="16" t="n"/>
+      <c r="C149" s="14" t="n"/>
       <c r="D149" s="6" t="n"/>
       <c r="E149" s="6" t="n"/>
       <c r="F149" s="6" t="n"/>
@@ -3660,7 +3442,7 @@
     <row r="150">
       <c r="A150" s="6" t="n"/>
       <c r="B150" s="6" t="n"/>
-      <c r="C150" s="16" t="n"/>
+      <c r="C150" s="14" t="n"/>
       <c r="D150" s="6" t="n"/>
       <c r="E150" s="6" t="n"/>
       <c r="F150" s="6" t="n"/>
@@ -3672,7 +3454,7 @@
     <row r="151">
       <c r="A151" s="6" t="n"/>
       <c r="B151" s="6" t="n"/>
-      <c r="C151" s="16" t="n"/>
+      <c r="C151" s="14" t="n"/>
       <c r="D151" s="6" t="n"/>
       <c r="E151" s="6" t="n"/>
       <c r="F151" s="6" t="n"/>
@@ -3684,7 +3466,7 @@
     <row r="152">
       <c r="A152" s="6" t="n"/>
       <c r="B152" s="6" t="n"/>
-      <c r="C152" s="16" t="n"/>
+      <c r="C152" s="14" t="n"/>
       <c r="D152" s="6" t="n"/>
       <c r="E152" s="6" t="n"/>
       <c r="F152" s="6" t="n"/>
@@ -3696,7 +3478,7 @@
     <row r="153">
       <c r="A153" s="6" t="n"/>
       <c r="B153" s="6" t="n"/>
-      <c r="C153" s="16" t="n"/>
+      <c r="C153" s="14" t="n"/>
       <c r="D153" s="6" t="n"/>
       <c r="E153" s="6" t="n"/>
       <c r="F153" s="6" t="n"/>
@@ -3708,7 +3490,7 @@
     <row r="154">
       <c r="A154" s="6" t="n"/>
       <c r="B154" s="6" t="n"/>
-      <c r="C154" s="16" t="n"/>
+      <c r="C154" s="14" t="n"/>
       <c r="D154" s="6" t="n"/>
       <c r="E154" s="6" t="n"/>
       <c r="F154" s="6" t="n"/>
@@ -3720,7 +3502,7 @@
     <row r="155">
       <c r="A155" s="6" t="n"/>
       <c r="B155" s="6" t="n"/>
-      <c r="C155" s="16" t="n"/>
+      <c r="C155" s="14" t="n"/>
       <c r="D155" s="6" t="n"/>
       <c r="E155" s="6" t="n"/>
       <c r="F155" s="6" t="n"/>
@@ -3732,7 +3514,7 @@
     <row r="156">
       <c r="A156" s="6" t="n"/>
       <c r="B156" s="6" t="n"/>
-      <c r="C156" s="16" t="n"/>
+      <c r="C156" s="14" t="n"/>
       <c r="D156" s="6" t="n"/>
       <c r="E156" s="6" t="n"/>
       <c r="F156" s="6" t="n"/>
@@ -3744,7 +3526,7 @@
     <row r="157">
       <c r="A157" s="6" t="n"/>
       <c r="B157" s="6" t="n"/>
-      <c r="C157" s="16" t="n"/>
+      <c r="C157" s="14" t="n"/>
       <c r="D157" s="6" t="n"/>
       <c r="E157" s="6" t="n"/>
       <c r="F157" s="6" t="n"/>
@@ -3756,7 +3538,7 @@
     <row r="158">
       <c r="A158" s="6" t="n"/>
       <c r="B158" s="6" t="n"/>
-      <c r="C158" s="16" t="n"/>
+      <c r="C158" s="14" t="n"/>
       <c r="D158" s="6" t="n"/>
       <c r="E158" s="6" t="n"/>
       <c r="F158" s="6" t="n"/>
@@ -3768,7 +3550,7 @@
     <row r="159">
       <c r="A159" s="6" t="n"/>
       <c r="B159" s="6" t="n"/>
-      <c r="C159" s="16" t="n"/>
+      <c r="C159" s="14" t="n"/>
       <c r="D159" s="6" t="n"/>
       <c r="E159" s="6" t="n"/>
       <c r="F159" s="6" t="n"/>
@@ -3780,7 +3562,7 @@
     <row r="160">
       <c r="A160" s="6" t="n"/>
       <c r="B160" s="6" t="n"/>
-      <c r="C160" s="16" t="n"/>
+      <c r="C160" s="14" t="n"/>
       <c r="D160" s="6" t="n"/>
       <c r="E160" s="6" t="n"/>
       <c r="F160" s="6" t="n"/>
@@ -3792,7 +3574,7 @@
     <row r="161">
       <c r="A161" s="6" t="n"/>
       <c r="B161" s="6" t="n"/>
-      <c r="C161" s="16" t="n"/>
+      <c r="C161" s="14" t="n"/>
       <c r="D161" s="6" t="n"/>
       <c r="E161" s="6" t="n"/>
       <c r="F161" s="6" t="n"/>
@@ -3804,7 +3586,7 @@
     <row r="162">
       <c r="A162" s="6" t="n"/>
       <c r="B162" s="6" t="n"/>
-      <c r="C162" s="16" t="n"/>
+      <c r="C162" s="14" t="n"/>
       <c r="D162" s="6" t="n"/>
       <c r="E162" s="6" t="n"/>
       <c r="F162" s="6" t="n"/>
@@ -3816,7 +3598,7 @@
     <row r="163">
       <c r="A163" s="6" t="n"/>
       <c r="B163" s="6" t="n"/>
-      <c r="C163" s="16" t="n"/>
+      <c r="C163" s="14" t="n"/>
       <c r="D163" s="6" t="n"/>
       <c r="E163" s="6" t="n"/>
       <c r="F163" s="6" t="n"/>
@@ -3828,7 +3610,7 @@
     <row r="164">
       <c r="A164" s="6" t="n"/>
       <c r="B164" s="6" t="n"/>
-      <c r="C164" s="16" t="n"/>
+      <c r="C164" s="14" t="n"/>
       <c r="D164" s="6" t="n"/>
       <c r="E164" s="6" t="n"/>
       <c r="F164" s="6" t="n"/>
@@ -3840,7 +3622,7 @@
     <row r="165">
       <c r="A165" s="6" t="n"/>
       <c r="B165" s="6" t="n"/>
-      <c r="C165" s="16" t="n"/>
+      <c r="C165" s="14" t="n"/>
       <c r="D165" s="6" t="n"/>
       <c r="E165" s="6" t="n"/>
       <c r="F165" s="6" t="n"/>
@@ -3852,7 +3634,7 @@
     <row r="166">
       <c r="A166" s="6" t="n"/>
       <c r="B166" s="6" t="n"/>
-      <c r="C166" s="16" t="n"/>
+      <c r="C166" s="14" t="n"/>
       <c r="D166" s="6" t="n"/>
       <c r="E166" s="6" t="n"/>
       <c r="F166" s="6" t="n"/>
@@ -3864,7 +3646,7 @@
     <row r="167">
       <c r="A167" s="6" t="n"/>
       <c r="B167" s="6" t="n"/>
-      <c r="C167" s="16" t="n"/>
+      <c r="C167" s="14" t="n"/>
       <c r="D167" s="6" t="n"/>
       <c r="E167" s="6" t="n"/>
       <c r="F167" s="6" t="n"/>
@@ -3876,7 +3658,7 @@
     <row r="168">
       <c r="A168" s="6" t="n"/>
       <c r="B168" s="6" t="n"/>
-      <c r="C168" s="16" t="n"/>
+      <c r="C168" s="14" t="n"/>
       <c r="D168" s="6" t="n"/>
       <c r="E168" s="6" t="n"/>
       <c r="F168" s="6" t="n"/>
@@ -3888,7 +3670,7 @@
     <row r="169">
       <c r="A169" s="6" t="n"/>
       <c r="B169" s="6" t="n"/>
-      <c r="C169" s="16" t="n"/>
+      <c r="C169" s="14" t="n"/>
       <c r="D169" s="6" t="n"/>
       <c r="E169" s="6" t="n"/>
       <c r="F169" s="6" t="n"/>
@@ -3900,7 +3682,7 @@
     <row r="170">
       <c r="A170" s="6" t="n"/>
       <c r="B170" s="6" t="n"/>
-      <c r="C170" s="16" t="n"/>
+      <c r="C170" s="14" t="n"/>
       <c r="D170" s="6" t="n"/>
       <c r="E170" s="6" t="n"/>
       <c r="F170" s="6" t="n"/>
@@ -3912,7 +3694,7 @@
     <row r="171">
       <c r="A171" s="6" t="n"/>
       <c r="B171" s="6" t="n"/>
-      <c r="C171" s="16" t="n"/>
+      <c r="C171" s="14" t="n"/>
       <c r="D171" s="6" t="n"/>
       <c r="E171" s="6" t="n"/>
       <c r="F171" s="6" t="n"/>
@@ -3924,7 +3706,7 @@
     <row r="172">
       <c r="A172" s="6" t="n"/>
       <c r="B172" s="6" t="n"/>
-      <c r="C172" s="16" t="n"/>
+      <c r="C172" s="14" t="n"/>
       <c r="D172" s="6" t="n"/>
       <c r="E172" s="6" t="n"/>
       <c r="F172" s="6" t="n"/>
@@ -3936,7 +3718,7 @@
     <row r="173">
       <c r="A173" s="6" t="n"/>
       <c r="B173" s="6" t="n"/>
-      <c r="C173" s="16" t="n"/>
+      <c r="C173" s="14" t="n"/>
       <c r="D173" s="6" t="n"/>
       <c r="E173" s="6" t="n"/>
       <c r="F173" s="6" t="n"/>
@@ -3948,7 +3730,7 @@
     <row r="174">
       <c r="A174" s="6" t="n"/>
       <c r="B174" s="6" t="n"/>
-      <c r="C174" s="16" t="n"/>
+      <c r="C174" s="14" t="n"/>
       <c r="D174" s="6" t="n"/>
       <c r="E174" s="6" t="n"/>
       <c r="F174" s="6" t="n"/>
@@ -3960,7 +3742,7 @@
     <row r="175">
       <c r="A175" s="6" t="n"/>
       <c r="B175" s="6" t="n"/>
-      <c r="C175" s="16" t="n"/>
+      <c r="C175" s="14" t="n"/>
       <c r="D175" s="6" t="n"/>
       <c r="E175" s="6" t="n"/>
       <c r="F175" s="6" t="n"/>
@@ -3972,7 +3754,7 @@
     <row r="176">
       <c r="A176" s="6" t="n"/>
       <c r="B176" s="6" t="n"/>
-      <c r="C176" s="16" t="n"/>
+      <c r="C176" s="14" t="n"/>
       <c r="D176" s="6" t="n"/>
       <c r="E176" s="6" t="n"/>
       <c r="F176" s="6" t="n"/>
@@ -3984,7 +3766,7 @@
     <row r="177">
       <c r="A177" s="6" t="n"/>
       <c r="B177" s="6" t="n"/>
-      <c r="C177" s="16" t="n"/>
+      <c r="C177" s="14" t="n"/>
       <c r="D177" s="6" t="n"/>
       <c r="E177" s="6" t="n"/>
       <c r="F177" s="6" t="n"/>
@@ -3996,7 +3778,7 @@
     <row r="178">
       <c r="A178" s="6" t="n"/>
       <c r="B178" s="6" t="n"/>
-      <c r="C178" s="16" t="n"/>
+      <c r="C178" s="14" t="n"/>
       <c r="D178" s="6" t="n"/>
       <c r="E178" s="6" t="n"/>
       <c r="F178" s="6" t="n"/>
@@ -4008,7 +3790,7 @@
     <row r="179">
       <c r="A179" s="6" t="n"/>
       <c r="B179" s="6" t="n"/>
-      <c r="C179" s="16" t="n"/>
+      <c r="C179" s="14" t="n"/>
       <c r="D179" s="6" t="n"/>
       <c r="E179" s="6" t="n"/>
       <c r="F179" s="6" t="n"/>
@@ -4020,7 +3802,7 @@
     <row r="180">
       <c r="A180" s="6" t="n"/>
       <c r="B180" s="6" t="n"/>
-      <c r="C180" s="16" t="n"/>
+      <c r="C180" s="14" t="n"/>
       <c r="D180" s="6" t="n"/>
       <c r="E180" s="6" t="n"/>
       <c r="F180" s="6" t="n"/>
@@ -4032,7 +3814,7 @@
     <row r="181">
       <c r="A181" s="6" t="n"/>
       <c r="B181" s="6" t="n"/>
-      <c r="C181" s="16" t="n"/>
+      <c r="C181" s="14" t="n"/>
       <c r="D181" s="6" t="n"/>
       <c r="E181" s="6" t="n"/>
       <c r="F181" s="6" t="n"/>
@@ -4044,7 +3826,7 @@
     <row r="182">
       <c r="A182" s="6" t="n"/>
       <c r="B182" s="6" t="n"/>
-      <c r="C182" s="16" t="n"/>
+      <c r="C182" s="14" t="n"/>
       <c r="D182" s="6" t="n"/>
       <c r="E182" s="6" t="n"/>
       <c r="F182" s="6" t="n"/>
@@ -4056,7 +3838,7 @@
     <row r="183">
       <c r="A183" s="6" t="n"/>
       <c r="B183" s="6" t="n"/>
-      <c r="C183" s="16" t="n"/>
+      <c r="C183" s="14" t="n"/>
       <c r="D183" s="6" t="n"/>
       <c r="E183" s="6" t="n"/>
       <c r="F183" s="6" t="n"/>
@@ -4068,7 +3850,7 @@
     <row r="184">
       <c r="A184" s="6" t="n"/>
       <c r="B184" s="6" t="n"/>
-      <c r="C184" s="16" t="n"/>
+      <c r="C184" s="14" t="n"/>
       <c r="D184" s="6" t="n"/>
       <c r="E184" s="6" t="n"/>
       <c r="F184" s="6" t="n"/>
@@ -4080,7 +3862,7 @@
     <row r="185">
       <c r="A185" s="6" t="n"/>
       <c r="B185" s="6" t="n"/>
-      <c r="C185" s="16" t="n"/>
+      <c r="C185" s="14" t="n"/>
       <c r="D185" s="6" t="n"/>
       <c r="E185" s="6" t="n"/>
       <c r="F185" s="6" t="n"/>
@@ -4092,7 +3874,7 @@
     <row r="186">
       <c r="A186" s="6" t="n"/>
       <c r="B186" s="6" t="n"/>
-      <c r="C186" s="16" t="n"/>
+      <c r="C186" s="14" t="n"/>
       <c r="D186" s="6" t="n"/>
       <c r="E186" s="6" t="n"/>
       <c r="F186" s="6" t="n"/>
@@ -4104,7 +3886,7 @@
     <row r="187">
       <c r="A187" s="6" t="n"/>
       <c r="B187" s="6" t="n"/>
-      <c r="C187" s="16" t="n"/>
+      <c r="C187" s="14" t="n"/>
       <c r="D187" s="6" t="n"/>
       <c r="E187" s="6" t="n"/>
       <c r="F187" s="6" t="n"/>
@@ -4116,7 +3898,7 @@
     <row r="188">
       <c r="A188" s="6" t="n"/>
       <c r="B188" s="6" t="n"/>
-      <c r="C188" s="16" t="n"/>
+      <c r="C188" s="14" t="n"/>
       <c r="D188" s="6" t="n"/>
       <c r="E188" s="6" t="n"/>
       <c r="F188" s="6" t="n"/>
@@ -4128,7 +3910,7 @@
     <row r="189">
       <c r="A189" s="6" t="n"/>
       <c r="B189" s="6" t="n"/>
-      <c r="C189" s="16" t="n"/>
+      <c r="C189" s="14" t="n"/>
       <c r="D189" s="6" t="n"/>
       <c r="E189" s="6" t="n"/>
       <c r="F189" s="6" t="n"/>
@@ -4140,7 +3922,7 @@
     <row r="190">
       <c r="A190" s="6" t="n"/>
       <c r="B190" s="6" t="n"/>
-      <c r="C190" s="16" t="n"/>
+      <c r="C190" s="14" t="n"/>
       <c r="D190" s="6" t="n"/>
       <c r="E190" s="6" t="n"/>
       <c r="F190" s="6" t="n"/>
@@ -4152,7 +3934,7 @@
     <row r="191">
       <c r="A191" s="6" t="n"/>
       <c r="B191" s="6" t="n"/>
-      <c r="C191" s="16" t="n"/>
+      <c r="C191" s="14" t="n"/>
       <c r="D191" s="6" t="n"/>
       <c r="E191" s="6" t="n"/>
       <c r="F191" s="6" t="n"/>
@@ -4164,7 +3946,7 @@
     <row r="192">
       <c r="A192" s="6" t="n"/>
       <c r="B192" s="6" t="n"/>
-      <c r="C192" s="16" t="n"/>
+      <c r="C192" s="14" t="n"/>
       <c r="D192" s="6" t="n"/>
       <c r="E192" s="6" t="n"/>
       <c r="F192" s="6" t="n"/>
@@ -4176,7 +3958,7 @@
     <row r="193">
       <c r="A193" s="6" t="n"/>
       <c r="B193" s="6" t="n"/>
-      <c r="C193" s="16" t="n"/>
+      <c r="C193" s="14" t="n"/>
       <c r="D193" s="6" t="n"/>
       <c r="E193" s="6" t="n"/>
       <c r="F193" s="6" t="n"/>
@@ -4188,7 +3970,7 @@
     <row r="194">
       <c r="A194" s="6" t="n"/>
       <c r="B194" s="6" t="n"/>
-      <c r="C194" s="16" t="n"/>
+      <c r="C194" s="14" t="n"/>
       <c r="D194" s="6" t="n"/>
       <c r="E194" s="6" t="n"/>
       <c r="F194" s="6" t="n"/>
@@ -4200,7 +3982,7 @@
     <row r="195">
       <c r="A195" s="6" t="n"/>
       <c r="B195" s="6" t="n"/>
-      <c r="C195" s="16" t="n"/>
+      <c r="C195" s="14" t="n"/>
       <c r="D195" s="6" t="n"/>
       <c r="E195" s="6" t="n"/>
       <c r="F195" s="6" t="n"/>
@@ -4212,7 +3994,7 @@
     <row r="196">
       <c r="A196" s="6" t="n"/>
       <c r="B196" s="6" t="n"/>
-      <c r="C196" s="16" t="n"/>
+      <c r="C196" s="14" t="n"/>
       <c r="D196" s="6" t="n"/>
       <c r="E196" s="6" t="n"/>
       <c r="F196" s="6" t="n"/>
@@ -4224,7 +4006,7 @@
     <row r="197">
       <c r="A197" s="6" t="n"/>
       <c r="B197" s="6" t="n"/>
-      <c r="C197" s="16" t="n"/>
+      <c r="C197" s="14" t="n"/>
       <c r="D197" s="6" t="n"/>
       <c r="E197" s="6" t="n"/>
       <c r="F197" s="6" t="n"/>
@@ -4236,7 +4018,7 @@
     <row r="198">
       <c r="A198" s="6" t="n"/>
       <c r="B198" s="6" t="n"/>
-      <c r="C198" s="16" t="n"/>
+      <c r="C198" s="14" t="n"/>
       <c r="D198" s="6" t="n"/>
       <c r="E198" s="6" t="n"/>
       <c r="F198" s="6" t="n"/>
@@ -4248,7 +4030,7 @@
     <row r="199">
       <c r="A199" s="6" t="n"/>
       <c r="B199" s="6" t="n"/>
-      <c r="C199" s="16" t="n"/>
+      <c r="C199" s="14" t="n"/>
       <c r="D199" s="6" t="n"/>
       <c r="E199" s="6" t="n"/>
       <c r="F199" s="6" t="n"/>
@@ -4260,7 +4042,7 @@
     <row r="200">
       <c r="A200" s="6" t="n"/>
       <c r="B200" s="6" t="n"/>
-      <c r="C200" s="16" t="n"/>
+      <c r="C200" s="14" t="n"/>
       <c r="D200" s="6" t="n"/>
       <c r="E200" s="6" t="n"/>
       <c r="F200" s="6" t="n"/>
@@ -4272,7 +4054,7 @@
     <row r="201">
       <c r="A201" s="6" t="n"/>
       <c r="B201" s="6" t="n"/>
-      <c r="C201" s="16" t="n"/>
+      <c r="C201" s="14" t="n"/>
       <c r="D201" s="6" t="n"/>
       <c r="E201" s="6" t="n"/>
       <c r="F201" s="6" t="n"/>
@@ -4284,7 +4066,7 @@
     <row r="202">
       <c r="A202" s="6" t="n"/>
       <c r="B202" s="6" t="n"/>
-      <c r="C202" s="16" t="n"/>
+      <c r="C202" s="14" t="n"/>
       <c r="D202" s="6" t="n"/>
       <c r="E202" s="6" t="n"/>
       <c r="F202" s="6" t="n"/>
@@ -4296,7 +4078,7 @@
     <row r="203">
       <c r="A203" s="6" t="n"/>
       <c r="B203" s="6" t="n"/>
-      <c r="C203" s="16" t="n"/>
+      <c r="C203" s="14" t="n"/>
       <c r="D203" s="6" t="n"/>
       <c r="E203" s="6" t="n"/>
       <c r="F203" s="6" t="n"/>
@@ -4308,7 +4090,7 @@
     <row r="204">
       <c r="A204" s="6" t="n"/>
       <c r="B204" s="6" t="n"/>
-      <c r="C204" s="16" t="n"/>
+      <c r="C204" s="14" t="n"/>
       <c r="D204" s="6" t="n"/>
       <c r="E204" s="6" t="n"/>
       <c r="F204" s="6" t="n"/>
@@ -4320,7 +4102,7 @@
     <row r="205">
       <c r="A205" s="6" t="n"/>
       <c r="B205" s="6" t="n"/>
-      <c r="C205" s="16" t="n"/>
+      <c r="C205" s="14" t="n"/>
       <c r="D205" s="6" t="n"/>
       <c r="E205" s="6" t="n"/>
       <c r="F205" s="6" t="n"/>
@@ -4332,7 +4114,7 @@
     <row r="206">
       <c r="A206" s="6" t="n"/>
       <c r="B206" s="6" t="n"/>
-      <c r="C206" s="16" t="n"/>
+      <c r="C206" s="14" t="n"/>
       <c r="D206" s="6" t="n"/>
       <c r="E206" s="6" t="n"/>
       <c r="F206" s="6" t="n"/>
@@ -4344,7 +4126,7 @@
     <row r="207">
       <c r="A207" s="6" t="n"/>
       <c r="B207" s="6" t="n"/>
-      <c r="C207" s="16" t="n"/>
+      <c r="C207" s="14" t="n"/>
       <c r="D207" s="6" t="n"/>
       <c r="E207" s="6" t="n"/>
       <c r="F207" s="6" t="n"/>
@@ -4356,7 +4138,7 @@
     <row r="208">
       <c r="A208" s="6" t="n"/>
       <c r="B208" s="6" t="n"/>
-      <c r="C208" s="16" t="n"/>
+      <c r="C208" s="14" t="n"/>
       <c r="D208" s="6" t="n"/>
       <c r="E208" s="6" t="n"/>
       <c r="F208" s="6" t="n"/>
@@ -4368,7 +4150,7 @@
     <row r="209">
       <c r="A209" s="6" t="n"/>
       <c r="B209" s="6" t="n"/>
-      <c r="C209" s="16" t="n"/>
+      <c r="C209" s="14" t="n"/>
       <c r="D209" s="6" t="n"/>
       <c r="E209" s="6" t="n"/>
       <c r="F209" s="6" t="n"/>
@@ -4380,7 +4162,7 @@
     <row r="210">
       <c r="A210" s="6" t="n"/>
       <c r="B210" s="6" t="n"/>
-      <c r="C210" s="16" t="n"/>
+      <c r="C210" s="14" t="n"/>
       <c r="D210" s="6" t="n"/>
       <c r="E210" s="6" t="n"/>
       <c r="F210" s="6" t="n"/>
@@ -4392,7 +4174,7 @@
     <row r="211">
       <c r="A211" s="6" t="n"/>
       <c r="B211" s="6" t="n"/>
-      <c r="C211" s="16" t="n"/>
+      <c r="C211" s="14" t="n"/>
       <c r="D211" s="6" t="n"/>
       <c r="E211" s="6" t="n"/>
       <c r="F211" s="6" t="n"/>
@@ -4404,7 +4186,7 @@
     <row r="212">
       <c r="A212" s="6" t="n"/>
       <c r="B212" s="6" t="n"/>
-      <c r="C212" s="16" t="n"/>
+      <c r="C212" s="14" t="n"/>
       <c r="D212" s="6" t="n"/>
       <c r="E212" s="6" t="n"/>
       <c r="F212" s="6" t="n"/>
@@ -4416,7 +4198,7 @@
     <row r="213">
       <c r="A213" s="6" t="n"/>
       <c r="B213" s="6" t="n"/>
-      <c r="C213" s="16" t="n"/>
+      <c r="C213" s="14" t="n"/>
       <c r="D213" s="6" t="n"/>
       <c r="E213" s="6" t="n"/>
       <c r="F213" s="6" t="n"/>
@@ -4428,7 +4210,7 @@
     <row r="214">
       <c r="A214" s="6" t="n"/>
       <c r="B214" s="6" t="n"/>
-      <c r="C214" s="16" t="n"/>
+      <c r="C214" s="14" t="n"/>
       <c r="D214" s="6" t="n"/>
       <c r="E214" s="6" t="n"/>
       <c r="F214" s="6" t="n"/>
@@ -4440,7 +4222,7 @@
     <row r="215">
       <c r="A215" s="6" t="n"/>
       <c r="B215" s="6" t="n"/>
-      <c r="C215" s="16" t="n"/>
+      <c r="C215" s="14" t="n"/>
       <c r="D215" s="6" t="n"/>
       <c r="E215" s="6" t="n"/>
       <c r="F215" s="6" t="n"/>
@@ -4452,7 +4234,7 @@
     <row r="216">
       <c r="A216" s="6" t="n"/>
       <c r="B216" s="6" t="n"/>
-      <c r="C216" s="16" t="n"/>
+      <c r="C216" s="14" t="n"/>
       <c r="D216" s="6" t="n"/>
       <c r="E216" s="6" t="n"/>
       <c r="F216" s="6" t="n"/>
@@ -4464,7 +4246,7 @@
     <row r="217">
       <c r="A217" s="6" t="n"/>
       <c r="B217" s="6" t="n"/>
-      <c r="C217" s="16" t="n"/>
+      <c r="C217" s="14" t="n"/>
       <c r="D217" s="6" t="n"/>
       <c r="E217" s="6" t="n"/>
       <c r="F217" s="6" t="n"/>
@@ -4476,7 +4258,7 @@
     <row r="218">
       <c r="A218" s="6" t="n"/>
       <c r="B218" s="6" t="n"/>
-      <c r="C218" s="16" t="n"/>
+      <c r="C218" s="14" t="n"/>
       <c r="D218" s="6" t="n"/>
       <c r="E218" s="6" t="n"/>
       <c r="F218" s="6" t="n"/>
@@ -4488,7 +4270,7 @@
     <row r="219">
       <c r="A219" s="6" t="n"/>
       <c r="B219" s="6" t="n"/>
-      <c r="C219" s="16" t="n"/>
+      <c r="C219" s="14" t="n"/>
       <c r="D219" s="6" t="n"/>
       <c r="E219" s="6" t="n"/>
       <c r="F219" s="6" t="n"/>
@@ -4500,7 +4282,7 @@
     <row r="220">
       <c r="A220" s="6" t="n"/>
       <c r="B220" s="6" t="n"/>
-      <c r="C220" s="16" t="n"/>
+      <c r="C220" s="14" t="n"/>
       <c r="D220" s="6" t="n"/>
       <c r="E220" s="6" t="n"/>
       <c r="F220" s="6" t="n"/>
@@ -4512,7 +4294,7 @@
     <row r="221">
       <c r="A221" s="6" t="n"/>
       <c r="B221" s="6" t="n"/>
-      <c r="C221" s="16" t="n"/>
+      <c r="C221" s="14" t="n"/>
       <c r="D221" s="6" t="n"/>
       <c r="E221" s="6" t="n"/>
       <c r="F221" s="6" t="n"/>
@@ -4524,7 +4306,7 @@
     <row r="222">
       <c r="A222" s="6" t="n"/>
       <c r="B222" s="6" t="n"/>
-      <c r="C222" s="16" t="n"/>
+      <c r="C222" s="14" t="n"/>
       <c r="D222" s="6" t="n"/>
       <c r="E222" s="6" t="n"/>
       <c r="F222" s="6" t="n"/>
@@ -4536,7 +4318,7 @@
     <row r="223">
       <c r="A223" s="6" t="n"/>
       <c r="B223" s="6" t="n"/>
-      <c r="C223" s="16" t="n"/>
+      <c r="C223" s="14" t="n"/>
       <c r="D223" s="6" t="n"/>
       <c r="E223" s="6" t="n"/>
       <c r="F223" s="6" t="n"/>
@@ -4548,7 +4330,7 @@
     <row r="224">
       <c r="A224" s="6" t="n"/>
       <c r="B224" s="6" t="n"/>
-      <c r="C224" s="16" t="n"/>
+      <c r="C224" s="14" t="n"/>
       <c r="D224" s="6" t="n"/>
       <c r="E224" s="6" t="n"/>
       <c r="F224" s="6" t="n"/>
@@ -4560,7 +4342,7 @@
     <row r="225">
       <c r="A225" s="6" t="n"/>
       <c r="B225" s="6" t="n"/>
-      <c r="C225" s="16" t="n"/>
+      <c r="C225" s="14" t="n"/>
       <c r="D225" s="6" t="n"/>
       <c r="E225" s="6" t="n"/>
       <c r="F225" s="6" t="n"/>
@@ -4572,7 +4354,7 @@
     <row r="226">
       <c r="A226" s="6" t="n"/>
       <c r="B226" s="6" t="n"/>
-      <c r="C226" s="16" t="n"/>
+      <c r="C226" s="14" t="n"/>
       <c r="D226" s="6" t="n"/>
       <c r="E226" s="6" t="n"/>
       <c r="F226" s="6" t="n"/>
@@ -4584,7 +4366,7 @@
     <row r="227">
       <c r="A227" s="6" t="n"/>
       <c r="B227" s="6" t="n"/>
-      <c r="C227" s="16" t="n"/>
+      <c r="C227" s="14" t="n"/>
       <c r="D227" s="6" t="n"/>
       <c r="E227" s="6" t="n"/>
       <c r="F227" s="6" t="n"/>
@@ -4596,7 +4378,7 @@
     <row r="228">
       <c r="A228" s="6" t="n"/>
       <c r="B228" s="6" t="n"/>
-      <c r="C228" s="16" t="n"/>
+      <c r="C228" s="14" t="n"/>
       <c r="D228" s="6" t="n"/>
       <c r="E228" s="6" t="n"/>
       <c r="F228" s="6" t="n"/>
@@ -4608,7 +4390,7 @@
     <row r="229">
       <c r="A229" s="6" t="n"/>
       <c r="B229" s="6" t="n"/>
-      <c r="C229" s="16" t="n"/>
+      <c r="C229" s="14" t="n"/>
       <c r="D229" s="6" t="n"/>
       <c r="E229" s="6" t="n"/>
       <c r="F229" s="6" t="n"/>
@@ -4620,7 +4402,7 @@
     <row r="230">
       <c r="A230" s="6" t="n"/>
       <c r="B230" s="6" t="n"/>
-      <c r="C230" s="16" t="n"/>
+      <c r="C230" s="14" t="n"/>
       <c r="D230" s="6" t="n"/>
       <c r="E230" s="6" t="n"/>
       <c r="F230" s="6" t="n"/>
@@ -4632,7 +4414,7 @@
     <row r="231">
       <c r="A231" s="6" t="n"/>
       <c r="B231" s="6" t="n"/>
-      <c r="C231" s="16" t="n"/>
+      <c r="C231" s="14" t="n"/>
       <c r="D231" s="6" t="n"/>
       <c r="E231" s="6" t="n"/>
       <c r="F231" s="6" t="n"/>
@@ -4644,7 +4426,7 @@
     <row r="232">
       <c r="A232" s="6" t="n"/>
       <c r="B232" s="6" t="n"/>
-      <c r="C232" s="16" t="n"/>
+      <c r="C232" s="14" t="n"/>
       <c r="D232" s="6" t="n"/>
       <c r="E232" s="6" t="n"/>
       <c r="F232" s="6" t="n"/>
@@ -4656,7 +4438,7 @@
     <row r="233">
       <c r="A233" s="6" t="n"/>
       <c r="B233" s="6" t="n"/>
-      <c r="C233" s="16" t="n"/>
+      <c r="C233" s="14" t="n"/>
       <c r="D233" s="6" t="n"/>
       <c r="E233" s="6" t="n"/>
       <c r="F233" s="6" t="n"/>
@@ -4668,7 +4450,7 @@
     <row r="234">
       <c r="A234" s="6" t="n"/>
       <c r="B234" s="6" t="n"/>
-      <c r="C234" s="16" t="n"/>
+      <c r="C234" s="14" t="n"/>
       <c r="D234" s="6" t="n"/>
       <c r="E234" s="6" t="n"/>
       <c r="F234" s="6" t="n"/>
@@ -4680,7 +4462,7 @@
     <row r="235">
       <c r="A235" s="6" t="n"/>
       <c r="B235" s="6" t="n"/>
-      <c r="C235" s="16" t="n"/>
+      <c r="C235" s="14" t="n"/>
       <c r="D235" s="6" t="n"/>
       <c r="E235" s="6" t="n"/>
       <c r="F235" s="6" t="n"/>
@@ -4692,7 +4474,7 @@
     <row r="236">
       <c r="A236" s="6" t="n"/>
       <c r="B236" s="6" t="n"/>
-      <c r="C236" s="16" t="n"/>
+      <c r="C236" s="14" t="n"/>
       <c r="D236" s="6" t="n"/>
       <c r="E236" s="6" t="n"/>
       <c r="F236" s="6" t="n"/>
@@ -4704,7 +4486,7 @@
     <row r="237">
       <c r="A237" s="6" t="n"/>
       <c r="B237" s="6" t="n"/>
-      <c r="C237" s="16" t="n"/>
+      <c r="C237" s="14" t="n"/>
       <c r="D237" s="6" t="n"/>
       <c r="E237" s="6" t="n"/>
       <c r="F237" s="6" t="n"/>
@@ -4716,7 +4498,7 @@
     <row r="238">
       <c r="A238" s="6" t="n"/>
       <c r="B238" s="6" t="n"/>
-      <c r="C238" s="16" t="n"/>
+      <c r="C238" s="14" t="n"/>
       <c r="D238" s="6" t="n"/>
       <c r="E238" s="6" t="n"/>
       <c r="F238" s="6" t="n"/>
@@ -4728,7 +4510,7 @@
     <row r="239">
       <c r="A239" s="6" t="n"/>
       <c r="B239" s="6" t="n"/>
-      <c r="C239" s="16" t="n"/>
+      <c r="C239" s="14" t="n"/>
       <c r="D239" s="6" t="n"/>
       <c r="E239" s="6" t="n"/>
       <c r="F239" s="6" t="n"/>
@@ -4740,7 +4522,7 @@
     <row r="240">
       <c r="A240" s="6" t="n"/>
       <c r="B240" s="6" t="n"/>
-      <c r="C240" s="16" t="n"/>
+      <c r="C240" s="14" t="n"/>
       <c r="D240" s="6" t="n"/>
       <c r="E240" s="6" t="n"/>
       <c r="F240" s="6" t="n"/>
@@ -4752,7 +4534,7 @@
     <row r="241">
       <c r="A241" s="6" t="n"/>
       <c r="B241" s="6" t="n"/>
-      <c r="C241" s="16" t="n"/>
+      <c r="C241" s="14" t="n"/>
       <c r="D241" s="6" t="n"/>
       <c r="E241" s="6" t="n"/>
       <c r="F241" s="6" t="n"/>
@@ -4764,7 +4546,7 @@
     <row r="242">
       <c r="A242" s="6" t="n"/>
       <c r="B242" s="6" t="n"/>
-      <c r="C242" s="16" t="n"/>
+      <c r="C242" s="14" t="n"/>
       <c r="D242" s="6" t="n"/>
       <c r="E242" s="6" t="n"/>
       <c r="F242" s="6" t="n"/>
@@ -4776,7 +4558,7 @@
     <row r="243">
       <c r="A243" s="6" t="n"/>
       <c r="B243" s="6" t="n"/>
-      <c r="C243" s="16" t="n"/>
+      <c r="C243" s="14" t="n"/>
       <c r="D243" s="6" t="n"/>
       <c r="E243" s="6" t="n"/>
       <c r="F243" s="6" t="n"/>
@@ -4788,7 +4570,7 @@
     <row r="244">
       <c r="A244" s="6" t="n"/>
       <c r="B244" s="6" t="n"/>
-      <c r="C244" s="16" t="n"/>
+      <c r="C244" s="14" t="n"/>
       <c r="D244" s="6" t="n"/>
       <c r="E244" s="6" t="n"/>
       <c r="F244" s="6" t="n"/>
@@ -4800,7 +4582,7 @@
     <row r="245">
       <c r="A245" s="6" t="n"/>
       <c r="B245" s="6" t="n"/>
-      <c r="C245" s="16" t="n"/>
+      <c r="C245" s="14" t="n"/>
       <c r="D245" s="6" t="n"/>
       <c r="E245" s="6" t="n"/>
       <c r="F245" s="6" t="n"/>
@@ -4812,7 +4594,7 @@
     <row r="246">
       <c r="A246" s="6" t="n"/>
       <c r="B246" s="6" t="n"/>
-      <c r="C246" s="16" t="n"/>
+      <c r="C246" s="14" t="n"/>
       <c r="D246" s="6" t="n"/>
       <c r="E246" s="6" t="n"/>
       <c r="F246" s="6" t="n"/>
@@ -4824,7 +4606,7 @@
     <row r="247">
       <c r="A247" s="6" t="n"/>
       <c r="B247" s="6" t="n"/>
-      <c r="C247" s="16" t="n"/>
+      <c r="C247" s="14" t="n"/>
       <c r="D247" s="6" t="n"/>
       <c r="E247" s="6" t="n"/>
       <c r="F247" s="6" t="n"/>
@@ -4836,7 +4618,7 @@
     <row r="248">
       <c r="A248" s="6" t="n"/>
       <c r="B248" s="6" t="n"/>
-      <c r="C248" s="16" t="n"/>
+      <c r="C248" s="14" t="n"/>
       <c r="D248" s="6" t="n"/>
       <c r="E248" s="6" t="n"/>
       <c r="F248" s="6" t="n"/>
@@ -4848,7 +4630,7 @@
     <row r="249">
       <c r="A249" s="6" t="n"/>
       <c r="B249" s="6" t="n"/>
-      <c r="C249" s="16" t="n"/>
+      <c r="C249" s="14" t="n"/>
       <c r="D249" s="6" t="n"/>
       <c r="E249" s="6" t="n"/>
       <c r="F249" s="6" t="n"/>
@@ -4860,7 +4642,7 @@
     <row r="250">
       <c r="A250" s="6" t="n"/>
       <c r="B250" s="6" t="n"/>
-      <c r="C250" s="16" t="n"/>
+      <c r="C250" s="14" t="n"/>
       <c r="D250" s="6" t="n"/>
       <c r="E250" s="6" t="n"/>
       <c r="F250" s="6" t="n"/>
@@ -4872,7 +4654,7 @@
     <row r="251">
       <c r="A251" s="6" t="n"/>
       <c r="B251" s="6" t="n"/>
-      <c r="C251" s="16" t="n"/>
+      <c r="C251" s="14" t="n"/>
       <c r="D251" s="6" t="n"/>
       <c r="E251" s="6" t="n"/>
       <c r="F251" s="6" t="n"/>
@@ -4884,7 +4666,7 @@
     <row r="252">
       <c r="A252" s="6" t="n"/>
       <c r="B252" s="6" t="n"/>
-      <c r="C252" s="16" t="n"/>
+      <c r="C252" s="14" t="n"/>
       <c r="D252" s="6" t="n"/>
       <c r="E252" s="6" t="n"/>
       <c r="F252" s="6" t="n"/>
@@ -4896,7 +4678,7 @@
     <row r="253">
       <c r="A253" s="6" t="n"/>
       <c r="B253" s="6" t="n"/>
-      <c r="C253" s="16" t="n"/>
+      <c r="C253" s="14" t="n"/>
       <c r="D253" s="6" t="n"/>
       <c r="E253" s="6" t="n"/>
       <c r="F253" s="6" t="n"/>
@@ -4908,7 +4690,7 @@
     <row r="254">
       <c r="A254" s="6" t="n"/>
       <c r="B254" s="6" t="n"/>
-      <c r="C254" s="16" t="n"/>
+      <c r="C254" s="14" t="n"/>
       <c r="D254" s="6" t="n"/>
       <c r="E254" s="6" t="n"/>
       <c r="F254" s="6" t="n"/>
@@ -4920,7 +4702,7 @@
     <row r="255">
       <c r="A255" s="6" t="n"/>
       <c r="B255" s="6" t="n"/>
-      <c r="C255" s="16" t="n"/>
+      <c r="C255" s="14" t="n"/>
       <c r="D255" s="6" t="n"/>
       <c r="E255" s="6" t="n"/>
       <c r="F255" s="6" t="n"/>
@@ -4932,7 +4714,7 @@
     <row r="256">
       <c r="A256" s="6" t="n"/>
       <c r="B256" s="6" t="n"/>
-      <c r="C256" s="16" t="n"/>
+      <c r="C256" s="14" t="n"/>
       <c r="D256" s="6" t="n"/>
       <c r="E256" s="6" t="n"/>
       <c r="F256" s="6" t="n"/>
@@ -4944,7 +4726,7 @@
     <row r="257">
       <c r="A257" s="6" t="n"/>
       <c r="B257" s="6" t="n"/>
-      <c r="C257" s="16" t="n"/>
+      <c r="C257" s="14" t="n"/>
       <c r="D257" s="6" t="n"/>
       <c r="E257" s="6" t="n"/>
       <c r="F257" s="6" t="n"/>
@@ -4956,7 +4738,7 @@
     <row r="258">
       <c r="A258" s="6" t="n"/>
       <c r="B258" s="6" t="n"/>
-      <c r="C258" s="16" t="n"/>
+      <c r="C258" s="14" t="n"/>
       <c r="D258" s="6" t="n"/>
       <c r="E258" s="6" t="n"/>
       <c r="F258" s="6" t="n"/>
@@ -4968,7 +4750,7 @@
     <row r="259">
       <c r="A259" s="6" t="n"/>
       <c r="B259" s="6" t="n"/>
-      <c r="C259" s="16" t="n"/>
+      <c r="C259" s="14" t="n"/>
       <c r="D259" s="6" t="n"/>
       <c r="E259" s="6" t="n"/>
       <c r="F259" s="6" t="n"/>
@@ -4980,7 +4762,7 @@
     <row r="260">
       <c r="A260" s="6" t="n"/>
       <c r="B260" s="6" t="n"/>
-      <c r="C260" s="16" t="n"/>
+      <c r="C260" s="14" t="n"/>
       <c r="D260" s="6" t="n"/>
       <c r="E260" s="6" t="n"/>
       <c r="F260" s="6" t="n"/>
@@ -4992,7 +4774,7 @@
     <row r="261">
       <c r="A261" s="6" t="n"/>
       <c r="B261" s="6" t="n"/>
-      <c r="C261" s="16" t="n"/>
+      <c r="C261" s="14" t="n"/>
       <c r="D261" s="6" t="n"/>
       <c r="E261" s="6" t="n"/>
       <c r="F261" s="6" t="n"/>
@@ -5004,7 +4786,7 @@
     <row r="262">
       <c r="A262" s="6" t="n"/>
       <c r="B262" s="6" t="n"/>
-      <c r="C262" s="16" t="n"/>
+      <c r="C262" s="14" t="n"/>
       <c r="D262" s="6" t="n"/>
       <c r="E262" s="6" t="n"/>
       <c r="F262" s="6" t="n"/>
@@ -5016,7 +4798,7 @@
     <row r="263">
       <c r="A263" s="6" t="n"/>
       <c r="B263" s="6" t="n"/>
-      <c r="C263" s="16" t="n"/>
+      <c r="C263" s="14" t="n"/>
       <c r="D263" s="6" t="n"/>
       <c r="E263" s="6" t="n"/>
       <c r="F263" s="6" t="n"/>
@@ -5028,7 +4810,7 @@
     <row r="264">
       <c r="A264" s="6" t="n"/>
       <c r="B264" s="6" t="n"/>
-      <c r="C264" s="16" t="n"/>
+      <c r="C264" s="14" t="n"/>
       <c r="D264" s="6" t="n"/>
       <c r="E264" s="6" t="n"/>
       <c r="F264" s="6" t="n"/>
@@ -5040,7 +4822,7 @@
     <row r="265">
       <c r="A265" s="6" t="n"/>
       <c r="B265" s="6" t="n"/>
-      <c r="C265" s="16" t="n"/>
+      <c r="C265" s="14" t="n"/>
       <c r="D265" s="6" t="n"/>
       <c r="E265" s="6" t="n"/>
       <c r="F265" s="6" t="n"/>
@@ -5052,7 +4834,7 @@
     <row r="266">
       <c r="A266" s="6" t="n"/>
       <c r="B266" s="6" t="n"/>
-      <c r="C266" s="16" t="n"/>
+      <c r="C266" s="14" t="n"/>
       <c r="D266" s="6" t="n"/>
       <c r="E266" s="6" t="n"/>
       <c r="F266" s="6" t="n"/>
@@ -5064,7 +4846,7 @@
     <row r="267">
       <c r="A267" s="6" t="n"/>
       <c r="B267" s="6" t="n"/>
-      <c r="C267" s="16" t="n"/>
+      <c r="C267" s="14" t="n"/>
       <c r="D267" s="6" t="n"/>
       <c r="E267" s="6" t="n"/>
       <c r="F267" s="6" t="n"/>
@@ -5076,7 +4858,7 @@
     <row r="268">
       <c r="A268" s="6" t="n"/>
       <c r="B268" s="6" t="n"/>
-      <c r="C268" s="16" t="n"/>
+      <c r="C268" s="14" t="n"/>
       <c r="D268" s="6" t="n"/>
       <c r="E268" s="6" t="n"/>
       <c r="F268" s="6" t="n"/>
@@ -5088,7 +4870,7 @@
     <row r="269">
       <c r="A269" s="6" t="n"/>
       <c r="B269" s="6" t="n"/>
-      <c r="C269" s="16" t="n"/>
+      <c r="C269" s="14" t="n"/>
       <c r="D269" s="6" t="n"/>
       <c r="E269" s="6" t="n"/>
       <c r="F269" s="6" t="n"/>
@@ -5100,7 +4882,7 @@
     <row r="270">
       <c r="A270" s="6" t="n"/>
       <c r="B270" s="6" t="n"/>
-      <c r="C270" s="16" t="n"/>
+      <c r="C270" s="14" t="n"/>
       <c r="D270" s="6" t="n"/>
       <c r="E270" s="6" t="n"/>
       <c r="F270" s="6" t="n"/>
@@ -5112,7 +4894,7 @@
     <row r="271">
       <c r="A271" s="6" t="n"/>
       <c r="B271" s="6" t="n"/>
-      <c r="C271" s="16" t="n"/>
+      <c r="C271" s="14" t="n"/>
       <c r="D271" s="6" t="n"/>
       <c r="E271" s="6" t="n"/>
       <c r="F271" s="6" t="n"/>
@@ -5124,7 +4906,7 @@
     <row r="272">
       <c r="A272" s="6" t="n"/>
       <c r="B272" s="6" t="n"/>
-      <c r="C272" s="16" t="n"/>
+      <c r="C272" s="14" t="n"/>
       <c r="D272" s="6" t="n"/>
       <c r="E272" s="6" t="n"/>
       <c r="F272" s="6" t="n"/>
@@ -5136,7 +4918,7 @@
     <row r="273">
       <c r="A273" s="6" t="n"/>
       <c r="B273" s="6" t="n"/>
-      <c r="C273" s="16" t="n"/>
+      <c r="C273" s="14" t="n"/>
       <c r="D273" s="6" t="n"/>
       <c r="E273" s="6" t="n"/>
       <c r="F273" s="6" t="n"/>
@@ -5148,7 +4930,7 @@
     <row r="274">
       <c r="A274" s="6" t="n"/>
       <c r="B274" s="6" t="n"/>
-      <c r="C274" s="16" t="n"/>
+      <c r="C274" s="14" t="n"/>
       <c r="D274" s="6" t="n"/>
       <c r="E274" s="6" t="n"/>
       <c r="F274" s="6" t="n"/>
@@ -5160,7 +4942,7 @@
     <row r="275">
       <c r="A275" s="6" t="n"/>
       <c r="B275" s="6" t="n"/>
-      <c r="C275" s="16" t="n"/>
+      <c r="C275" s="14" t="n"/>
       <c r="D275" s="6" t="n"/>
       <c r="E275" s="6" t="n"/>
       <c r="F275" s="6" t="n"/>
@@ -5172,7 +4954,7 @@
     <row r="276">
       <c r="A276" s="6" t="n"/>
       <c r="B276" s="6" t="n"/>
-      <c r="C276" s="16" t="n"/>
+      <c r="C276" s="14" t="n"/>
       <c r="D276" s="6" t="n"/>
       <c r="E276" s="6" t="n"/>
       <c r="F276" s="6" t="n"/>
@@ -5184,7 +4966,7 @@
     <row r="277">
       <c r="A277" s="6" t="n"/>
       <c r="B277" s="6" t="n"/>
-      <c r="C277" s="16" t="n"/>
+      <c r="C277" s="14" t="n"/>
       <c r="D277" s="6" t="n"/>
       <c r="E277" s="6" t="n"/>
       <c r="F277" s="6" t="n"/>
@@ -5196,7 +4978,7 @@
     <row r="278">
       <c r="A278" s="6" t="n"/>
       <c r="B278" s="6" t="n"/>
-      <c r="C278" s="16" t="n"/>
+      <c r="C278" s="14" t="n"/>
       <c r="D278" s="6" t="n"/>
       <c r="E278" s="6" t="n"/>
       <c r="F278" s="6" t="n"/>
@@ -5208,7 +4990,7 @@
     <row r="279">
       <c r="A279" s="6" t="n"/>
       <c r="B279" s="6" t="n"/>
-      <c r="C279" s="16" t="n"/>
+      <c r="C279" s="14" t="n"/>
       <c r="D279" s="6" t="n"/>
       <c r="E279" s="6" t="n"/>
       <c r="F279" s="6" t="n"/>
@@ -5220,7 +5002,7 @@
     <row r="280">
       <c r="A280" s="6" t="n"/>
       <c r="B280" s="6" t="n"/>
-      <c r="C280" s="16" t="n"/>
+      <c r="C280" s="14" t="n"/>
       <c r="D280" s="6" t="n"/>
       <c r="E280" s="6" t="n"/>
       <c r="F280" s="6" t="n"/>
@@ -5232,7 +5014,7 @@
     <row r="281">
       <c r="A281" s="6" t="n"/>
       <c r="B281" s="6" t="n"/>
-      <c r="C281" s="16" t="n"/>
+      <c r="C281" s="14" t="n"/>
       <c r="D281" s="6" t="n"/>
       <c r="E281" s="6" t="n"/>
       <c r="F281" s="6" t="n"/>
@@ -5244,7 +5026,7 @@
     <row r="282">
       <c r="A282" s="6" t="n"/>
       <c r="B282" s="6" t="n"/>
-      <c r="C282" s="16" t="n"/>
+      <c r="C282" s="14" t="n"/>
       <c r="D282" s="6" t="n"/>
       <c r="E282" s="6" t="n"/>
       <c r="F282" s="6" t="n"/>
@@ -5256,7 +5038,7 @@
     <row r="283">
       <c r="A283" s="6" t="n"/>
       <c r="B283" s="6" t="n"/>
-      <c r="C283" s="16" t="n"/>
+      <c r="C283" s="14" t="n"/>
       <c r="D283" s="6" t="n"/>
       <c r="E283" s="6" t="n"/>
       <c r="F283" s="6" t="n"/>
@@ -5268,7 +5050,7 @@
     <row r="284">
       <c r="A284" s="6" t="n"/>
       <c r="B284" s="6" t="n"/>
-      <c r="C284" s="16" t="n"/>
+      <c r="C284" s="14" t="n"/>
       <c r="D284" s="6" t="n"/>
       <c r="E284" s="6" t="n"/>
       <c r="F284" s="6" t="n"/>
@@ -5280,7 +5062,7 @@
     <row r="285">
       <c r="A285" s="6" t="n"/>
       <c r="B285" s="6" t="n"/>
-      <c r="C285" s="16" t="n"/>
+      <c r="C285" s="14" t="n"/>
       <c r="D285" s="6" t="n"/>
       <c r="E285" s="6" t="n"/>
       <c r="F285" s="6" t="n"/>
@@ -5292,7 +5074,7 @@
     <row r="286">
       <c r="A286" s="6" t="n"/>
       <c r="B286" s="6" t="n"/>
-      <c r="C286" s="16" t="n"/>
+      <c r="C286" s="14" t="n"/>
       <c r="D286" s="6" t="n"/>
       <c r="E286" s="6" t="n"/>
       <c r="F286" s="6" t="n"/>
@@ -5304,7 +5086,7 @@
     <row r="287">
       <c r="A287" s="6" t="n"/>
       <c r="B287" s="6" t="n"/>
-      <c r="C287" s="16" t="n"/>
+      <c r="C287" s="14" t="n"/>
       <c r="D287" s="6" t="n"/>
       <c r="E287" s="6" t="n"/>
       <c r="F287" s="6" t="n"/>
@@ -5316,7 +5098,7 @@
     <row r="288">
       <c r="A288" s="6" t="n"/>
       <c r="B288" s="6" t="n"/>
-      <c r="C288" s="16" t="n"/>
+      <c r="C288" s="14" t="n"/>
       <c r="D288" s="6" t="n"/>
       <c r="E288" s="6" t="n"/>
       <c r="F288" s="6" t="n"/>
@@ -5328,7 +5110,7 @@
     <row r="289">
       <c r="A289" s="6" t="n"/>
       <c r="B289" s="6" t="n"/>
-      <c r="C289" s="16" t="n"/>
+      <c r="C289" s="14" t="n"/>
       <c r="D289" s="6" t="n"/>
       <c r="E289" s="6" t="n"/>
       <c r="F289" s="6" t="n"/>
@@ -5340,7 +5122,7 @@
     <row r="290">
       <c r="A290" s="6" t="n"/>
       <c r="B290" s="6" t="n"/>
-      <c r="C290" s="16" t="n"/>
+      <c r="C290" s="14" t="n"/>
       <c r="D290" s="6" t="n"/>
       <c r="E290" s="6" t="n"/>
       <c r="F290" s="6" t="n"/>
@@ -5352,7 +5134,7 @@
     <row r="291">
       <c r="A291" s="6" t="n"/>
       <c r="B291" s="6" t="n"/>
-      <c r="C291" s="16" t="n"/>
+      <c r="C291" s="14" t="n"/>
       <c r="D291" s="6" t="n"/>
       <c r="E291" s="6" t="n"/>
       <c r="F291" s="6" t="n"/>
@@ -5364,7 +5146,7 @@
     <row r="292">
       <c r="A292" s="6" t="n"/>
       <c r="B292" s="6" t="n"/>
-      <c r="C292" s="16" t="n"/>
+      <c r="C292" s="14" t="n"/>
       <c r="D292" s="6" t="n"/>
       <c r="E292" s="6" t="n"/>
       <c r="F292" s="6" t="n"/>
@@ -5376,7 +5158,7 @@
     <row r="293">
       <c r="A293" s="6" t="n"/>
       <c r="B293" s="6" t="n"/>
-      <c r="C293" s="16" t="n"/>
+      <c r="C293" s="14" t="n"/>
       <c r="D293" s="6" t="n"/>
       <c r="E293" s="6" t="n"/>
       <c r="F293" s="6" t="n"/>
@@ -5388,7 +5170,7 @@
     <row r="294">
       <c r="A294" s="6" t="n"/>
       <c r="B294" s="6" t="n"/>
-      <c r="C294" s="16" t="n"/>
+      <c r="C294" s="14" t="n"/>
       <c r="D294" s="6" t="n"/>
       <c r="E294" s="6" t="n"/>
       <c r="F294" s="6" t="n"/>
@@ -5400,7 +5182,7 @@
     <row r="295">
       <c r="A295" s="6" t="n"/>
       <c r="B295" s="6" t="n"/>
-      <c r="C295" s="16" t="n"/>
+      <c r="C295" s="14" t="n"/>
       <c r="D295" s="6" t="n"/>
       <c r="E295" s="6" t="n"/>
       <c r="F295" s="6" t="n"/>
@@ -5412,7 +5194,7 @@
     <row r="296">
       <c r="A296" s="6" t="n"/>
       <c r="B296" s="6" t="n"/>
-      <c r="C296" s="16" t="n"/>
+      <c r="C296" s="14" t="n"/>
       <c r="D296" s="6" t="n"/>
       <c r="E296" s="6" t="n"/>
       <c r="F296" s="6" t="n"/>
@@ -5424,7 +5206,7 @@
     <row r="297">
       <c r="A297" s="6" t="n"/>
       <c r="B297" s="6" t="n"/>
-      <c r="C297" s="16" t="n"/>
+      <c r="C297" s="14" t="n"/>
       <c r="D297" s="6" t="n"/>
       <c r="E297" s="6" t="n"/>
       <c r="F297" s="6" t="n"/>
@@ -5436,7 +5218,7 @@
     <row r="298">
       <c r="A298" s="6" t="n"/>
       <c r="B298" s="6" t="n"/>
-      <c r="C298" s="16" t="n"/>
+      <c r="C298" s="14" t="n"/>
       <c r="D298" s="6" t="n"/>
       <c r="E298" s="6" t="n"/>
       <c r="F298" s="6" t="n"/>
@@ -5448,7 +5230,7 @@
     <row r="299">
       <c r="A299" s="6" t="n"/>
       <c r="B299" s="6" t="n"/>
-      <c r="C299" s="16" t="n"/>
+      <c r="C299" s="14" t="n"/>
       <c r="D299" s="6" t="n"/>
       <c r="E299" s="6" t="n"/>
       <c r="F299" s="6" t="n"/>

</xml_diff>